<commit_message>
Auto sync Onetech 28/10/2026 17:30
</commit_message>
<xml_diff>
--- a/data/Thang10/DANH_SACH_KET_QUA_CUA_HANG_THAM_GIA_CHUONG_TRINH.xlsx
+++ b/data/Thang10/DANH_SACH_KET_QUA_CUA_HANG_THAM_GIA_CHUONG_TRINH.xlsx
@@ -2713,6 +2713,51 @@
     <t>Active</t>
   </si>
   <si>
+    <t>999754600</t>
+  </si>
+  <si>
+    <t>Chị Loan</t>
+  </si>
+  <si>
+    <t>6/2, Đường Số 6</t>
+  </si>
+  <si>
+    <t>999762653</t>
+  </si>
+  <si>
+    <t>Cà Phê Thúy Vy</t>
+  </si>
+  <si>
+    <t>Số 1351, Đường Nguyễn Thị Định</t>
+  </si>
+  <si>
+    <t>999765789</t>
+  </si>
+  <si>
+    <t>TH Hoa Phượng</t>
+  </si>
+  <si>
+    <t>34/33, Đường Số 2</t>
+  </si>
+  <si>
+    <t>2344002</t>
+  </si>
+  <si>
+    <t>Thịnh Thoa</t>
+  </si>
+  <si>
+    <t>34, Đường 4</t>
+  </si>
+  <si>
+    <t>2004898</t>
+  </si>
+  <si>
+    <t>Tạp Hóa Kim Thoa</t>
+  </si>
+  <si>
+    <t>40 Cảng Phú Hữu, Nguyễn Duy Trinh</t>
+  </si>
+  <si>
     <t>3362</t>
   </si>
   <si>
@@ -2722,51 +2767,6 @@
     <t>107, Lò Lu</t>
   </si>
   <si>
-    <t>999754600</t>
-  </si>
-  <si>
-    <t>Chị Loan</t>
-  </si>
-  <si>
-    <t>6/2, Đường Số 6</t>
-  </si>
-  <si>
-    <t>999762653</t>
-  </si>
-  <si>
-    <t>Cà Phê Thúy Vy</t>
-  </si>
-  <si>
-    <t>Số 1351, Đường Nguyễn Thị Định</t>
-  </si>
-  <si>
-    <t>999765789</t>
-  </si>
-  <si>
-    <t>TH Hoa Phượng</t>
-  </si>
-  <si>
-    <t>34/33, Đường Số 2</t>
-  </si>
-  <si>
-    <t>2344002</t>
-  </si>
-  <si>
-    <t>Thịnh Thoa</t>
-  </si>
-  <si>
-    <t>34, Đường 4</t>
-  </si>
-  <si>
-    <t>2004898</t>
-  </si>
-  <si>
-    <t>Tạp Hóa Kim Thoa</t>
-  </si>
-  <si>
-    <t>40 Cảng Phú Hữu, Nguyễn Duy Trinh</t>
-  </si>
-  <si>
     <t>1-6JP933U</t>
   </si>
   <si>
@@ -2878,6 +2878,48 @@
     <t>MSC_BEV_Chương trình TBTN_Tủ mát Nước giải khát_HCM_All2026_T10</t>
   </si>
   <si>
+    <t>2432200</t>
+  </si>
+  <si>
+    <t>G-Net Tycoon</t>
+  </si>
+  <si>
+    <t>Số 117A, Đường 39</t>
+  </si>
+  <si>
+    <t>2451874</t>
+  </si>
+  <si>
+    <t>Quán Cơm Bảo An</t>
+  </si>
+  <si>
+    <t>242, Đường 57 - CL</t>
+  </si>
+  <si>
+    <t>3136368</t>
+  </si>
+  <si>
+    <t>Chợ Sạch 24H</t>
+  </si>
+  <si>
+    <t>35 Đường Số 12, Bưng Ông Thoàn</t>
+  </si>
+  <si>
+    <t>3063948</t>
+  </si>
+  <si>
+    <t>Cà Phê Chị Tuyết</t>
+  </si>
+  <si>
+    <t>Đối Diện Cổng E, Đường Số 57 CL</t>
+  </si>
+  <si>
+    <t>2894640</t>
+  </si>
+  <si>
+    <t>Mino Mart</t>
+  </si>
+  <si>
     <t>2128924</t>
   </si>
   <si>
@@ -2887,46 +2929,13 @@
     <t>22/10 Đường 990, Nguyễn Duy Trinh</t>
   </si>
   <si>
-    <t>2432200</t>
-  </si>
-  <si>
-    <t>G-Net Tycoon</t>
-  </si>
-  <si>
-    <t>Số 117A, Đường 39</t>
-  </si>
-  <si>
-    <t>2451874</t>
-  </si>
-  <si>
-    <t>Quán Cơm Bảo An</t>
-  </si>
-  <si>
-    <t>242, Đường 57 - CL</t>
-  </si>
-  <si>
-    <t>2894640</t>
-  </si>
-  <si>
-    <t>Mino Mart</t>
-  </si>
-  <si>
-    <t>3063948</t>
-  </si>
-  <si>
-    <t>Cà Phê Chị Tuyết</t>
-  </si>
-  <si>
-    <t>Đối Diện Cổng E, Đường Số 57 CL</t>
-  </si>
-  <si>
-    <t>3136368</t>
-  </si>
-  <si>
-    <t>Chợ Sạch 24H</t>
-  </si>
-  <si>
-    <t>35 Đường Số 12, Bưng Ông Thoàn</t>
+    <t>999191040</t>
+  </si>
+  <si>
+    <t>Tạp Hóa Sáu Tèo</t>
+  </si>
+  <si>
+    <t>250, Trường Lưu</t>
   </si>
   <si>
     <t>999115327</t>
@@ -2936,15 +2945,6 @@
   </si>
   <si>
     <t>Số 313, Lê Văn Thịnh</t>
-  </si>
-  <si>
-    <t>999191040</t>
-  </si>
-  <si>
-    <t>Tạp Hóa Sáu Tèo</t>
-  </si>
-  <si>
-    <t>250, Trường Lưu</t>
   </si>
   <si>
     <t>999210374</t>
@@ -42092,16 +42092,16 @@
         <v>50</v>
       </c>
       <c r="M311" s="3" t="s">
-        <v>115</v>
+        <v>62</v>
       </c>
       <c r="N311" s="3" t="s">
-        <v>116</v>
+        <v>63</v>
       </c>
       <c r="O311" s="3" t="s">
-        <v>117</v>
+        <v>64</v>
       </c>
       <c r="P311" s="3" t="s">
-        <v>118</v>
+        <v>65</v>
       </c>
       <c r="Q311" s="3" t="s">
         <v>46</v>
@@ -42134,7 +42134,7 @@
         <v>10</v>
       </c>
       <c r="AA311" s="7">
-        <v>10</v>
+        <v>10.75</v>
       </c>
       <c r="AB311" s="7">
         <v>1</v>
@@ -42164,7 +42164,7 @@
         <v>58</v>
       </c>
       <c r="AK311" s="6">
-        <v>46298.66540524305</v>
+        <v>46312.58308098379</v>
       </c>
       <c r="AL311" s="3" t="s">
         <v>46</v>
@@ -42176,7 +42176,7 @@
         <v>58</v>
       </c>
       <c r="AO311" s="6">
-        <v>46298.66540524305</v>
+        <v>46312.58308098379</v>
       </c>
     </row>
     <row r="312" spans="1:41" x14ac:dyDescent="0.25">
@@ -42217,16 +42217,16 @@
         <v>50</v>
       </c>
       <c r="M312" s="3" t="s">
-        <v>62</v>
+        <v>105</v>
       </c>
       <c r="N312" s="3" t="s">
-        <v>63</v>
+        <v>106</v>
       </c>
       <c r="O312" s="3" t="s">
-        <v>64</v>
+        <v>107</v>
       </c>
       <c r="P312" s="3" t="s">
-        <v>65</v>
+        <v>108</v>
       </c>
       <c r="Q312" s="3" t="s">
         <v>46</v>
@@ -42259,7 +42259,7 @@
         <v>10</v>
       </c>
       <c r="AA312" s="7">
-        <v>10.75</v>
+        <v>10</v>
       </c>
       <c r="AB312" s="7">
         <v>1</v>
@@ -42289,7 +42289,7 @@
         <v>58</v>
       </c>
       <c r="AK312" s="6">
-        <v>46312.58308098379</v>
+        <v>46310.439036655094</v>
       </c>
       <c r="AL312" s="3" t="s">
         <v>46</v>
@@ -42301,7 +42301,7 @@
         <v>58</v>
       </c>
       <c r="AO312" s="6">
-        <v>46312.58308098379</v>
+        <v>46310.439036655094</v>
       </c>
     </row>
     <row r="313" spans="1:41" x14ac:dyDescent="0.25">
@@ -42342,16 +42342,16 @@
         <v>50</v>
       </c>
       <c r="M313" s="3" t="s">
-        <v>105</v>
+        <v>115</v>
       </c>
       <c r="N313" s="3" t="s">
-        <v>106</v>
+        <v>116</v>
       </c>
       <c r="O313" s="3" t="s">
-        <v>107</v>
+        <v>117</v>
       </c>
       <c r="P313" s="3" t="s">
-        <v>108</v>
+        <v>118</v>
       </c>
       <c r="Q313" s="3" t="s">
         <v>46</v>
@@ -42414,7 +42414,7 @@
         <v>58</v>
       </c>
       <c r="AK313" s="6">
-        <v>46310.439036655094</v>
+        <v>46301.30899568287</v>
       </c>
       <c r="AL313" s="3" t="s">
         <v>46</v>
@@ -42426,7 +42426,7 @@
         <v>58</v>
       </c>
       <c r="AO313" s="6">
-        <v>46310.439036655094</v>
+        <v>46301.30899568287</v>
       </c>
     </row>
     <row r="314" spans="1:41" x14ac:dyDescent="0.25">
@@ -42455,28 +42455,28 @@
         <v>45</v>
       </c>
       <c r="I314" s="3" t="s">
-        <v>909</v>
+        <v>271</v>
       </c>
       <c r="J314" s="3" t="s">
-        <v>910</v>
+        <v>272</v>
       </c>
       <c r="K314" s="3" t="s">
-        <v>911</v>
+        <v>273</v>
       </c>
       <c r="L314" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M314" s="3" t="s">
-        <v>115</v>
+        <v>79</v>
       </c>
       <c r="N314" s="3" t="s">
-        <v>116</v>
+        <v>80</v>
       </c>
       <c r="O314" s="3" t="s">
-        <v>117</v>
+        <v>81</v>
       </c>
       <c r="P314" s="3" t="s">
-        <v>118</v>
+        <v>82</v>
       </c>
       <c r="Q314" s="3" t="s">
         <v>46</v>
@@ -42539,7 +42539,7 @@
         <v>58</v>
       </c>
       <c r="AK314" s="6">
-        <v>46301.30899568287</v>
+        <v>46301.5776272338</v>
       </c>
       <c r="AL314" s="3" t="s">
         <v>46</v>
@@ -42551,7 +42551,7 @@
         <v>58</v>
       </c>
       <c r="AO314" s="6">
-        <v>46301.30899568287</v>
+        <v>46301.5776272338</v>
       </c>
     </row>
     <row r="315" spans="1:41" x14ac:dyDescent="0.25">
@@ -42580,28 +42580,28 @@
         <v>45</v>
       </c>
       <c r="I315" s="3" t="s">
-        <v>271</v>
+        <v>322</v>
       </c>
       <c r="J315" s="3" t="s">
-        <v>272</v>
+        <v>323</v>
       </c>
       <c r="K315" s="3" t="s">
-        <v>273</v>
+        <v>324</v>
       </c>
       <c r="L315" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M315" s="3" t="s">
-        <v>79</v>
+        <v>105</v>
       </c>
       <c r="N315" s="3" t="s">
-        <v>80</v>
+        <v>106</v>
       </c>
       <c r="O315" s="3" t="s">
-        <v>81</v>
+        <v>107</v>
       </c>
       <c r="P315" s="3" t="s">
-        <v>82</v>
+        <v>108</v>
       </c>
       <c r="Q315" s="3" t="s">
         <v>46</v>
@@ -42634,7 +42634,7 @@
         <v>10</v>
       </c>
       <c r="AA315" s="7">
-        <v>10</v>
+        <v>10.5</v>
       </c>
       <c r="AB315" s="7">
         <v>1</v>
@@ -42664,7 +42664,7 @@
         <v>58</v>
       </c>
       <c r="AK315" s="6">
-        <v>46301.5776272338</v>
+        <v>46303.59483915509</v>
       </c>
       <c r="AL315" s="3" t="s">
         <v>46</v>
@@ -42676,7 +42676,7 @@
         <v>58</v>
       </c>
       <c r="AO315" s="6">
-        <v>46301.5776272338</v>
+        <v>46303.59483915509</v>
       </c>
     </row>
     <row r="316" spans="1:41" x14ac:dyDescent="0.25">
@@ -42705,28 +42705,28 @@
         <v>45</v>
       </c>
       <c r="I316" s="3" t="s">
-        <v>322</v>
+        <v>150</v>
       </c>
       <c r="J316" s="3" t="s">
-        <v>323</v>
+        <v>151</v>
       </c>
       <c r="K316" s="3" t="s">
-        <v>324</v>
+        <v>152</v>
       </c>
       <c r="L316" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M316" s="3" t="s">
-        <v>105</v>
+        <v>153</v>
       </c>
       <c r="N316" s="3" t="s">
-        <v>106</v>
+        <v>154</v>
       </c>
       <c r="O316" s="3" t="s">
-        <v>107</v>
+        <v>155</v>
       </c>
       <c r="P316" s="3" t="s">
-        <v>108</v>
+        <v>156</v>
       </c>
       <c r="Q316" s="3" t="s">
         <v>46</v>
@@ -42759,7 +42759,7 @@
         <v>10</v>
       </c>
       <c r="AA316" s="7">
-        <v>10.5</v>
+        <v>10</v>
       </c>
       <c r="AB316" s="7">
         <v>1</v>
@@ -42789,7 +42789,7 @@
         <v>58</v>
       </c>
       <c r="AK316" s="6">
-        <v>46303.59483915509</v>
+        <v>46298.66540524305</v>
       </c>
       <c r="AL316" s="3" t="s">
         <v>46</v>
@@ -42801,7 +42801,7 @@
         <v>58</v>
       </c>
       <c r="AO316" s="6">
-        <v>46303.59483915509</v>
+        <v>46298.66540524305</v>
       </c>
     </row>
     <row r="317" spans="1:41" x14ac:dyDescent="0.25">
@@ -42830,28 +42830,28 @@
         <v>45</v>
       </c>
       <c r="I317" s="3" t="s">
-        <v>150</v>
+        <v>909</v>
       </c>
       <c r="J317" s="3" t="s">
-        <v>151</v>
+        <v>910</v>
       </c>
       <c r="K317" s="3" t="s">
-        <v>152</v>
+        <v>911</v>
       </c>
       <c r="L317" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M317" s="3" t="s">
-        <v>153</v>
+        <v>115</v>
       </c>
       <c r="N317" s="3" t="s">
-        <v>154</v>
+        <v>116</v>
       </c>
       <c r="O317" s="3" t="s">
-        <v>155</v>
+        <v>117</v>
       </c>
       <c r="P317" s="3" t="s">
-        <v>156</v>
+        <v>118</v>
       </c>
       <c r="Q317" s="3" t="s">
         <v>46</v>
@@ -42967,16 +42967,16 @@
         <v>50</v>
       </c>
       <c r="M318" s="3" t="s">
-        <v>115</v>
+        <v>131</v>
       </c>
       <c r="N318" s="3" t="s">
-        <v>116</v>
+        <v>132</v>
       </c>
       <c r="O318" s="3" t="s">
-        <v>117</v>
+        <v>133</v>
       </c>
       <c r="P318" s="3" t="s">
-        <v>118</v>
+        <v>134</v>
       </c>
       <c r="Q318" s="3" t="s">
         <v>46</v>
@@ -43039,7 +43039,7 @@
         <v>58</v>
       </c>
       <c r="AK318" s="6">
-        <v>46298.66540524305</v>
+        <v>46316.79383703704</v>
       </c>
       <c r="AL318" s="3" t="s">
         <v>46</v>
@@ -43051,7 +43051,7 @@
         <v>58</v>
       </c>
       <c r="AO318" s="6">
-        <v>46298.66540524305</v>
+        <v>46316.79383703704</v>
       </c>
     </row>
     <row r="319" spans="1:41" x14ac:dyDescent="0.25">
@@ -43080,28 +43080,28 @@
         <v>45</v>
       </c>
       <c r="I319" s="3" t="s">
-        <v>915</v>
+        <v>138</v>
       </c>
       <c r="J319" s="3" t="s">
-        <v>916</v>
+        <v>139</v>
       </c>
       <c r="K319" s="3" t="s">
-        <v>917</v>
+        <v>140</v>
       </c>
       <c r="L319" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M319" s="3" t="s">
-        <v>131</v>
+        <v>105</v>
       </c>
       <c r="N319" s="3" t="s">
-        <v>132</v>
+        <v>106</v>
       </c>
       <c r="O319" s="3" t="s">
-        <v>133</v>
+        <v>107</v>
       </c>
       <c r="P319" s="3" t="s">
-        <v>134</v>
+        <v>108</v>
       </c>
       <c r="Q319" s="3" t="s">
         <v>46</v>
@@ -43134,7 +43134,7 @@
         <v>10</v>
       </c>
       <c r="AA319" s="7">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="AB319" s="7">
         <v>1</v>
@@ -43164,7 +43164,7 @@
         <v>58</v>
       </c>
       <c r="AK319" s="6">
-        <v>46316.79383703704</v>
+        <v>46303.59483915509</v>
       </c>
       <c r="AL319" s="3" t="s">
         <v>46</v>
@@ -43176,7 +43176,7 @@
         <v>58</v>
       </c>
       <c r="AO319" s="6">
-        <v>46316.79383703704</v>
+        <v>46303.59483915509</v>
       </c>
     </row>
     <row r="320" spans="1:41" x14ac:dyDescent="0.25">
@@ -43205,28 +43205,28 @@
         <v>45</v>
       </c>
       <c r="I320" s="3" t="s">
-        <v>138</v>
+        <v>915</v>
       </c>
       <c r="J320" s="3" t="s">
-        <v>139</v>
+        <v>916</v>
       </c>
       <c r="K320" s="3" t="s">
-        <v>140</v>
+        <v>917</v>
       </c>
       <c r="L320" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M320" s="3" t="s">
-        <v>105</v>
+        <v>115</v>
       </c>
       <c r="N320" s="3" t="s">
-        <v>106</v>
+        <v>116</v>
       </c>
       <c r="O320" s="3" t="s">
-        <v>107</v>
+        <v>117</v>
       </c>
       <c r="P320" s="3" t="s">
-        <v>108</v>
+        <v>118</v>
       </c>
       <c r="Q320" s="3" t="s">
         <v>46</v>
@@ -43259,7 +43259,7 @@
         <v>10</v>
       </c>
       <c r="AA320" s="7">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="AB320" s="7">
         <v>1</v>
@@ -43289,7 +43289,7 @@
         <v>58</v>
       </c>
       <c r="AK320" s="6">
-        <v>46303.59483915509</v>
+        <v>46298.66540524305</v>
       </c>
       <c r="AL320" s="3" t="s">
         <v>46</v>
@@ -43301,7 +43301,7 @@
         <v>58</v>
       </c>
       <c r="AO320" s="6">
-        <v>46303.59483915509</v>
+        <v>46298.66540524305</v>
       </c>
     </row>
     <row r="321" spans="1:41" x14ac:dyDescent="0.25">
@@ -44854,13 +44854,13 @@
         <v>128</v>
       </c>
       <c r="Q333" s="5">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="R333" s="5">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="S333" s="5">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="T333" s="3" t="s">
         <v>894</v>
@@ -46229,13 +46229,13 @@
         <v>134</v>
       </c>
       <c r="Q344" s="5">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="R344" s="5">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="S344" s="5">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="T344" s="3" t="s">
         <v>894</v>
@@ -46455,37 +46455,37 @@
         <v>921</v>
       </c>
       <c r="I346" s="3" t="s">
-        <v>378</v>
+        <v>939</v>
       </c>
       <c r="J346" s="3" t="s">
-        <v>379</v>
+        <v>744</v>
       </c>
       <c r="K346" s="3" t="s">
-        <v>380</v>
+        <v>940</v>
       </c>
       <c r="L346" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M346" s="3" t="s">
-        <v>125</v>
+        <v>79</v>
       </c>
       <c r="N346" s="3" t="s">
-        <v>126</v>
+        <v>80</v>
       </c>
       <c r="O346" s="3" t="s">
-        <v>127</v>
+        <v>81</v>
       </c>
       <c r="P346" s="3" t="s">
-        <v>128</v>
+        <v>82</v>
       </c>
       <c r="Q346" s="5">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="R346" s="5">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="S346" s="5">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="T346" s="3" t="s">
         <v>894</v>
@@ -46509,7 +46509,7 @@
         <v>46</v>
       </c>
       <c r="AA346" s="7">
-        <v>156000</v>
+        <v>2416326</v>
       </c>
       <c r="AB346" s="7">
         <v>31</v>
@@ -46580,37 +46580,37 @@
         <v>921</v>
       </c>
       <c r="I347" s="3" t="s">
-        <v>939</v>
+        <v>948</v>
       </c>
       <c r="J347" s="3" t="s">
-        <v>744</v>
+        <v>949</v>
       </c>
       <c r="K347" s="3" t="s">
-        <v>940</v>
+        <v>950</v>
       </c>
       <c r="L347" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M347" s="3" t="s">
-        <v>79</v>
+        <v>131</v>
       </c>
       <c r="N347" s="3" t="s">
-        <v>80</v>
+        <v>132</v>
       </c>
       <c r="O347" s="3" t="s">
-        <v>81</v>
+        <v>133</v>
       </c>
       <c r="P347" s="3" t="s">
-        <v>82</v>
+        <v>134</v>
       </c>
       <c r="Q347" s="5">
-        <v>7</v>
+        <v>26</v>
       </c>
       <c r="R347" s="5">
-        <v>3</v>
+        <v>26</v>
       </c>
       <c r="S347" s="5">
-        <v>7</v>
+        <v>26</v>
       </c>
       <c r="T347" s="3" t="s">
         <v>894</v>
@@ -46634,7 +46634,7 @@
         <v>46</v>
       </c>
       <c r="AA347" s="7">
-        <v>2416326</v>
+        <v>2359523</v>
       </c>
       <c r="AB347" s="7">
         <v>31</v>
@@ -46705,37 +46705,37 @@
         <v>921</v>
       </c>
       <c r="I348" s="3" t="s">
-        <v>948</v>
+        <v>755</v>
       </c>
       <c r="J348" s="3" t="s">
-        <v>949</v>
+        <v>756</v>
       </c>
       <c r="K348" s="3" t="s">
-        <v>950</v>
+        <v>757</v>
       </c>
       <c r="L348" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M348" s="3" t="s">
-        <v>131</v>
+        <v>115</v>
       </c>
       <c r="N348" s="3" t="s">
-        <v>132</v>
+        <v>116</v>
       </c>
       <c r="O348" s="3" t="s">
-        <v>133</v>
+        <v>117</v>
       </c>
       <c r="P348" s="3" t="s">
-        <v>134</v>
+        <v>118</v>
       </c>
       <c r="Q348" s="5">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="R348" s="5">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="S348" s="5">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="T348" s="3" t="s">
         <v>894</v>
@@ -46759,7 +46759,7 @@
         <v>46</v>
       </c>
       <c r="AA348" s="7">
-        <v>2359523</v>
+        <v>2580460</v>
       </c>
       <c r="AB348" s="7">
         <v>31</v>
@@ -46830,37 +46830,37 @@
         <v>921</v>
       </c>
       <c r="I349" s="3" t="s">
-        <v>755</v>
+        <v>464</v>
       </c>
       <c r="J349" s="3" t="s">
-        <v>756</v>
+        <v>465</v>
       </c>
       <c r="K349" s="3" t="s">
-        <v>757</v>
+        <v>466</v>
       </c>
       <c r="L349" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M349" s="3" t="s">
-        <v>115</v>
+        <v>125</v>
       </c>
       <c r="N349" s="3" t="s">
-        <v>116</v>
+        <v>126</v>
       </c>
       <c r="O349" s="3" t="s">
-        <v>117</v>
+        <v>127</v>
       </c>
       <c r="P349" s="3" t="s">
-        <v>118</v>
+        <v>128</v>
       </c>
       <c r="Q349" s="5">
-        <v>13</v>
+        <v>34</v>
       </c>
       <c r="R349" s="5">
-        <v>13</v>
+        <v>34</v>
       </c>
       <c r="S349" s="5">
-        <v>13</v>
+        <v>34</v>
       </c>
       <c r="T349" s="3" t="s">
         <v>894</v>
@@ -46884,7 +46884,7 @@
         <v>46</v>
       </c>
       <c r="AA349" s="7">
-        <v>2580460</v>
+        <v>570000</v>
       </c>
       <c r="AB349" s="7">
         <v>31</v>
@@ -46955,13 +46955,13 @@
         <v>921</v>
       </c>
       <c r="I350" s="3" t="s">
-        <v>464</v>
+        <v>473</v>
       </c>
       <c r="J350" s="3" t="s">
-        <v>465</v>
+        <v>474</v>
       </c>
       <c r="K350" s="3" t="s">
-        <v>466</v>
+        <v>475</v>
       </c>
       <c r="L350" s="3" t="s">
         <v>50</v>
@@ -46979,13 +46979,13 @@
         <v>128</v>
       </c>
       <c r="Q350" s="5">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="R350" s="5">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="S350" s="5">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="T350" s="3" t="s">
         <v>894</v>
@@ -47009,7 +47009,7 @@
         <v>46</v>
       </c>
       <c r="AA350" s="7">
-        <v>570000</v>
+        <v>925650</v>
       </c>
       <c r="AB350" s="7">
         <v>31</v>
@@ -47080,13 +47080,13 @@
         <v>921</v>
       </c>
       <c r="I351" s="3" t="s">
-        <v>473</v>
+        <v>535</v>
       </c>
       <c r="J351" s="3" t="s">
-        <v>474</v>
+        <v>536</v>
       </c>
       <c r="K351" s="3" t="s">
-        <v>475</v>
+        <v>537</v>
       </c>
       <c r="L351" s="3" t="s">
         <v>50</v>
@@ -47104,13 +47104,13 @@
         <v>128</v>
       </c>
       <c r="Q351" s="5">
-        <v>28</v>
+        <v>5</v>
       </c>
       <c r="R351" s="5">
-        <v>28</v>
+        <v>3</v>
       </c>
       <c r="S351" s="5">
-        <v>28</v>
+        <v>6</v>
       </c>
       <c r="T351" s="3" t="s">
         <v>894</v>
@@ -47134,7 +47134,7 @@
         <v>46</v>
       </c>
       <c r="AA351" s="7">
-        <v>925650</v>
+        <v>590000</v>
       </c>
       <c r="AB351" s="7">
         <v>31</v>
@@ -47205,13 +47205,13 @@
         <v>921</v>
       </c>
       <c r="I352" s="3" t="s">
-        <v>535</v>
+        <v>575</v>
       </c>
       <c r="J352" s="3" t="s">
-        <v>536</v>
+        <v>576</v>
       </c>
       <c r="K352" s="3" t="s">
-        <v>537</v>
+        <v>577</v>
       </c>
       <c r="L352" s="3" t="s">
         <v>50</v>
@@ -47229,13 +47229,13 @@
         <v>128</v>
       </c>
       <c r="Q352" s="5">
-        <v>5</v>
+        <v>27</v>
       </c>
       <c r="R352" s="5">
-        <v>3</v>
+        <v>26</v>
       </c>
       <c r="S352" s="5">
-        <v>6</v>
+        <v>28</v>
       </c>
       <c r="T352" s="3" t="s">
         <v>894</v>
@@ -47259,7 +47259,7 @@
         <v>46</v>
       </c>
       <c r="AA352" s="7">
-        <v>590000</v>
+        <v>2566500</v>
       </c>
       <c r="AB352" s="7">
         <v>31</v>
@@ -47330,13 +47330,13 @@
         <v>921</v>
       </c>
       <c r="I353" s="3" t="s">
-        <v>575</v>
+        <v>578</v>
       </c>
       <c r="J353" s="3" t="s">
-        <v>576</v>
+        <v>579</v>
       </c>
       <c r="K353" s="3" t="s">
-        <v>577</v>
+        <v>580</v>
       </c>
       <c r="L353" s="3" t="s">
         <v>50</v>
@@ -47354,13 +47354,13 @@
         <v>128</v>
       </c>
       <c r="Q353" s="5">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="R353" s="5">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="S353" s="5">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="T353" s="3" t="s">
         <v>894</v>
@@ -47383,8 +47383,8 @@
       <c r="Z353" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="AA353" s="7">
-        <v>2566500</v>
+      <c r="AA353" s="3" t="s">
+        <v>46</v>
       </c>
       <c r="AB353" s="7">
         <v>31</v>
@@ -47455,37 +47455,37 @@
         <v>921</v>
       </c>
       <c r="I354" s="3" t="s">
-        <v>578</v>
+        <v>89</v>
       </c>
       <c r="J354" s="3" t="s">
-        <v>579</v>
+        <v>90</v>
       </c>
       <c r="K354" s="3" t="s">
-        <v>580</v>
+        <v>91</v>
       </c>
       <c r="L354" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M354" s="3" t="s">
-        <v>125</v>
+        <v>69</v>
       </c>
       <c r="N354" s="3" t="s">
-        <v>126</v>
+        <v>70</v>
       </c>
       <c r="O354" s="3" t="s">
-        <v>127</v>
+        <v>71</v>
       </c>
       <c r="P354" s="3" t="s">
-        <v>128</v>
+        <v>72</v>
       </c>
       <c r="Q354" s="5">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="R354" s="5">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="S354" s="5">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="T354" s="3" t="s">
         <v>894</v>
@@ -47508,8 +47508,8 @@
       <c r="Z354" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="AA354" s="3" t="s">
-        <v>46</v>
+      <c r="AA354" s="7">
+        <v>1246838</v>
       </c>
       <c r="AB354" s="7">
         <v>31</v>
@@ -47580,37 +47580,37 @@
         <v>921</v>
       </c>
       <c r="I355" s="3" t="s">
-        <v>659</v>
+        <v>699</v>
       </c>
       <c r="J355" s="3" t="s">
-        <v>660</v>
+        <v>700</v>
       </c>
       <c r="K355" s="3" t="s">
-        <v>661</v>
+        <v>701</v>
       </c>
       <c r="L355" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M355" s="3" t="s">
-        <v>125</v>
+        <v>115</v>
       </c>
       <c r="N355" s="3" t="s">
-        <v>126</v>
+        <v>116</v>
       </c>
       <c r="O355" s="3" t="s">
-        <v>127</v>
+        <v>117</v>
       </c>
       <c r="P355" s="3" t="s">
-        <v>128</v>
+        <v>118</v>
       </c>
       <c r="Q355" s="5">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="R355" s="5">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="S355" s="5">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="T355" s="3" t="s">
         <v>894</v>
@@ -47634,7 +47634,7 @@
         <v>46</v>
       </c>
       <c r="AA355" s="7">
-        <v>290939</v>
+        <v>339000</v>
       </c>
       <c r="AB355" s="7">
         <v>31</v>
@@ -47705,37 +47705,37 @@
         <v>921</v>
       </c>
       <c r="I356" s="3" t="s">
-        <v>89</v>
+        <v>659</v>
       </c>
       <c r="J356" s="3" t="s">
-        <v>90</v>
+        <v>660</v>
       </c>
       <c r="K356" s="3" t="s">
-        <v>91</v>
+        <v>661</v>
       </c>
       <c r="L356" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M356" s="3" t="s">
-        <v>69</v>
+        <v>125</v>
       </c>
       <c r="N356" s="3" t="s">
-        <v>70</v>
+        <v>126</v>
       </c>
       <c r="O356" s="3" t="s">
-        <v>71</v>
+        <v>127</v>
       </c>
       <c r="P356" s="3" t="s">
-        <v>72</v>
+        <v>128</v>
       </c>
       <c r="Q356" s="5">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="R356" s="5">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="S356" s="5">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="T356" s="3" t="s">
         <v>894</v>
@@ -47759,7 +47759,7 @@
         <v>46</v>
       </c>
       <c r="AA356" s="7">
-        <v>1246838</v>
+        <v>290939</v>
       </c>
       <c r="AB356" s="7">
         <v>31</v>
@@ -47830,37 +47830,37 @@
         <v>921</v>
       </c>
       <c r="I357" s="3" t="s">
-        <v>699</v>
+        <v>378</v>
       </c>
       <c r="J357" s="3" t="s">
-        <v>700</v>
+        <v>379</v>
       </c>
       <c r="K357" s="3" t="s">
-        <v>701</v>
+        <v>380</v>
       </c>
       <c r="L357" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M357" s="3" t="s">
-        <v>115</v>
+        <v>125</v>
       </c>
       <c r="N357" s="3" t="s">
-        <v>116</v>
+        <v>126</v>
       </c>
       <c r="O357" s="3" t="s">
-        <v>117</v>
+        <v>127</v>
       </c>
       <c r="P357" s="3" t="s">
-        <v>118</v>
+        <v>128</v>
       </c>
       <c r="Q357" s="5">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="R357" s="5">
-        <v>33</v>
+        <v>10</v>
       </c>
       <c r="S357" s="5">
-        <v>35</v>
+        <v>11</v>
       </c>
       <c r="T357" s="3" t="s">
         <v>894</v>
@@ -47884,7 +47884,7 @@
         <v>46</v>
       </c>
       <c r="AA357" s="7">
-        <v>339000</v>
+        <v>156000</v>
       </c>
       <c r="AB357" s="7">
         <v>31</v>
@@ -47955,13 +47955,13 @@
         <v>951</v>
       </c>
       <c r="I358" s="3" t="s">
-        <v>912</v>
+        <v>909</v>
       </c>
       <c r="J358" s="3" t="s">
-        <v>913</v>
+        <v>910</v>
       </c>
       <c r="K358" s="3" t="s">
-        <v>914</v>
+        <v>911</v>
       </c>
       <c r="L358" s="3" t="s">
         <v>50</v>
@@ -48092,22 +48092,22 @@
         <v>50</v>
       </c>
       <c r="M359" s="3" t="s">
-        <v>131</v>
+        <v>62</v>
       </c>
       <c r="N359" s="3" t="s">
-        <v>132</v>
+        <v>63</v>
       </c>
       <c r="O359" s="3" t="s">
-        <v>133</v>
+        <v>64</v>
       </c>
       <c r="P359" s="3" t="s">
-        <v>134</v>
+        <v>65</v>
       </c>
       <c r="Q359" s="5">
         <v>2</v>
       </c>
       <c r="R359" s="5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S359" s="5">
         <v>2</v>
@@ -48134,7 +48134,7 @@
         <v>46</v>
       </c>
       <c r="AA359" s="7">
-        <v>646676</v>
+        <v>1211240</v>
       </c>
       <c r="AB359" s="7">
         <v>1</v>
@@ -48205,37 +48205,37 @@
         <v>45</v>
       </c>
       <c r="I360" s="3" t="s">
-        <v>109</v>
+        <v>958</v>
       </c>
       <c r="J360" s="3" t="s">
-        <v>110</v>
+        <v>959</v>
       </c>
       <c r="K360" s="3" t="s">
-        <v>111</v>
+        <v>960</v>
       </c>
       <c r="L360" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M360" s="3" t="s">
-        <v>62</v>
+        <v>105</v>
       </c>
       <c r="N360" s="3" t="s">
-        <v>63</v>
+        <v>106</v>
       </c>
       <c r="O360" s="3" t="s">
-        <v>64</v>
+        <v>107</v>
       </c>
       <c r="P360" s="3" t="s">
-        <v>65</v>
+        <v>108</v>
       </c>
       <c r="Q360" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R360" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S360" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="T360" s="3" t="s">
         <v>894</v>
@@ -48259,7 +48259,7 @@
         <v>46</v>
       </c>
       <c r="AA360" s="7">
-        <v>558000</v>
+        <v>663000</v>
       </c>
       <c r="AB360" s="7">
         <v>1</v>
@@ -48286,10 +48286,10 @@
         <v>0</v>
       </c>
       <c r="AJ360" s="3" t="s">
-        <v>924</v>
+        <v>58</v>
       </c>
       <c r="AK360" s="6">
-        <v>46296.93825494213</v>
+        <v>46304.905077118055</v>
       </c>
       <c r="AL360" s="3" t="s">
         <v>46</v>
@@ -48298,10 +48298,10 @@
         <v>46</v>
       </c>
       <c r="AN360" s="3" t="s">
-        <v>924</v>
+        <v>58</v>
       </c>
       <c r="AO360" s="6">
-        <v>46296.93825494213</v>
+        <v>46304.905077118055</v>
       </c>
     </row>
     <row r="361" spans="1:41" x14ac:dyDescent="0.25">
@@ -48330,37 +48330,37 @@
         <v>45</v>
       </c>
       <c r="I361" s="3" t="s">
-        <v>135</v>
+        <v>286</v>
       </c>
       <c r="J361" s="3" t="s">
-        <v>136</v>
+        <v>287</v>
       </c>
       <c r="K361" s="3" t="s">
-        <v>137</v>
+        <v>288</v>
       </c>
       <c r="L361" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M361" s="3" t="s">
-        <v>131</v>
+        <v>105</v>
       </c>
       <c r="N361" s="3" t="s">
-        <v>132</v>
+        <v>106</v>
       </c>
       <c r="O361" s="3" t="s">
-        <v>133</v>
+        <v>107</v>
       </c>
       <c r="P361" s="3" t="s">
-        <v>134</v>
+        <v>108</v>
       </c>
       <c r="Q361" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R361" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S361" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="T361" s="3" t="s">
         <v>894</v>
@@ -48383,8 +48383,8 @@
       <c r="Z361" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="AA361" s="7">
-        <v>536250</v>
+      <c r="AA361" s="3" t="s">
+        <v>46</v>
       </c>
       <c r="AB361" s="7">
         <v>1</v>
@@ -48411,10 +48411,10 @@
         <v>0</v>
       </c>
       <c r="AJ361" s="3" t="s">
-        <v>924</v>
+        <v>58</v>
       </c>
       <c r="AK361" s="6">
-        <v>46296.93825494213</v>
+        <v>46301.927933530096</v>
       </c>
       <c r="AL361" s="3" t="s">
         <v>46</v>
@@ -48423,10 +48423,10 @@
         <v>46</v>
       </c>
       <c r="AN361" s="3" t="s">
-        <v>924</v>
+        <v>58</v>
       </c>
       <c r="AO361" s="6">
-        <v>46296.93825494213</v>
+        <v>46301.927933530096</v>
       </c>
     </row>
     <row r="362" spans="1:41" x14ac:dyDescent="0.25">
@@ -48455,28 +48455,28 @@
         <v>45</v>
       </c>
       <c r="I362" s="3" t="s">
-        <v>144</v>
+        <v>292</v>
       </c>
       <c r="J362" s="3" t="s">
-        <v>145</v>
+        <v>293</v>
       </c>
       <c r="K362" s="3" t="s">
-        <v>146</v>
+        <v>294</v>
       </c>
       <c r="L362" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M362" s="3" t="s">
-        <v>98</v>
+        <v>62</v>
       </c>
       <c r="N362" s="3" t="s">
-        <v>99</v>
+        <v>63</v>
       </c>
       <c r="O362" s="3" t="s">
-        <v>100</v>
+        <v>64</v>
       </c>
       <c r="P362" s="3" t="s">
-        <v>101</v>
+        <v>65</v>
       </c>
       <c r="Q362" s="5">
         <v>2</v>
@@ -48509,7 +48509,7 @@
         <v>46</v>
       </c>
       <c r="AA362" s="7">
-        <v>2736757</v>
+        <v>87000</v>
       </c>
       <c r="AB362" s="7">
         <v>1</v>
@@ -48580,28 +48580,28 @@
         <v>45</v>
       </c>
       <c r="I363" s="3" t="s">
-        <v>958</v>
+        <v>728</v>
       </c>
       <c r="J363" s="3" t="s">
-        <v>959</v>
+        <v>729</v>
       </c>
       <c r="K363" s="3" t="s">
-        <v>960</v>
+        <v>730</v>
       </c>
       <c r="L363" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M363" s="3" t="s">
-        <v>62</v>
+        <v>131</v>
       </c>
       <c r="N363" s="3" t="s">
-        <v>63</v>
+        <v>132</v>
       </c>
       <c r="O363" s="3" t="s">
-        <v>64</v>
+        <v>133</v>
       </c>
       <c r="P363" s="3" t="s">
-        <v>65</v>
+        <v>134</v>
       </c>
       <c r="Q363" s="5">
         <v>2</v>
@@ -48634,7 +48634,7 @@
         <v>46</v>
       </c>
       <c r="AA363" s="7">
-        <v>1211240</v>
+        <v>1567312</v>
       </c>
       <c r="AB363" s="7">
         <v>1</v>
@@ -48705,13 +48705,13 @@
         <v>45</v>
       </c>
       <c r="I364" s="3" t="s">
-        <v>961</v>
+        <v>322</v>
       </c>
       <c r="J364" s="3" t="s">
-        <v>962</v>
+        <v>323</v>
       </c>
       <c r="K364" s="3" t="s">
-        <v>963</v>
+        <v>324</v>
       </c>
       <c r="L364" s="3" t="s">
         <v>50</v>
@@ -48729,13 +48729,13 @@
         <v>108</v>
       </c>
       <c r="Q364" s="5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R364" s="5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S364" s="5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T364" s="3" t="s">
         <v>894</v>
@@ -48759,7 +48759,7 @@
         <v>46</v>
       </c>
       <c r="AA364" s="7">
-        <v>663000</v>
+        <v>5131620</v>
       </c>
       <c r="AB364" s="7">
         <v>1</v>
@@ -48786,10 +48786,10 @@
         <v>0</v>
       </c>
       <c r="AJ364" s="3" t="s">
-        <v>58</v>
+        <v>924</v>
       </c>
       <c r="AK364" s="6">
-        <v>46304.905077118055</v>
+        <v>46296.93825494213</v>
       </c>
       <c r="AL364" s="3" t="s">
         <v>46</v>
@@ -48798,10 +48798,10 @@
         <v>46</v>
       </c>
       <c r="AN364" s="3" t="s">
-        <v>58</v>
+        <v>924</v>
       </c>
       <c r="AO364" s="6">
-        <v>46304.905077118055</v>
+        <v>46296.93825494213</v>
       </c>
     </row>
     <row r="365" spans="1:41" x14ac:dyDescent="0.25">
@@ -48830,28 +48830,28 @@
         <v>45</v>
       </c>
       <c r="I365" s="3" t="s">
-        <v>722</v>
+        <v>422</v>
       </c>
       <c r="J365" s="3" t="s">
-        <v>723</v>
+        <v>423</v>
       </c>
       <c r="K365" s="3" t="s">
-        <v>724</v>
+        <v>424</v>
       </c>
       <c r="L365" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M365" s="3" t="s">
-        <v>62</v>
+        <v>131</v>
       </c>
       <c r="N365" s="3" t="s">
-        <v>63</v>
+        <v>132</v>
       </c>
       <c r="O365" s="3" t="s">
-        <v>64</v>
+        <v>133</v>
       </c>
       <c r="P365" s="3" t="s">
-        <v>65</v>
+        <v>134</v>
       </c>
       <c r="Q365" s="5">
         <v>2</v>
@@ -48884,7 +48884,7 @@
         <v>46</v>
       </c>
       <c r="AA365" s="7">
-        <v>1227480</v>
+        <v>698000</v>
       </c>
       <c r="AB365" s="7">
         <v>1</v>
@@ -48955,37 +48955,37 @@
         <v>45</v>
       </c>
       <c r="I366" s="3" t="s">
-        <v>286</v>
+        <v>772</v>
       </c>
       <c r="J366" s="3" t="s">
-        <v>287</v>
+        <v>773</v>
       </c>
       <c r="K366" s="3" t="s">
-        <v>288</v>
+        <v>774</v>
       </c>
       <c r="L366" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M366" s="3" t="s">
-        <v>105</v>
+        <v>62</v>
       </c>
       <c r="N366" s="3" t="s">
-        <v>106</v>
+        <v>63</v>
       </c>
       <c r="O366" s="3" t="s">
-        <v>107</v>
+        <v>64</v>
       </c>
       <c r="P366" s="3" t="s">
-        <v>108</v>
+        <v>65</v>
       </c>
       <c r="Q366" s="5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R366" s="5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S366" s="5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T366" s="3" t="s">
         <v>894</v>
@@ -49008,8 +49008,8 @@
       <c r="Z366" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="AA366" s="3" t="s">
-        <v>46</v>
+      <c r="AA366" s="7">
+        <v>2482921</v>
       </c>
       <c r="AB366" s="7">
         <v>1</v>
@@ -49036,10 +49036,10 @@
         <v>0</v>
       </c>
       <c r="AJ366" s="3" t="s">
-        <v>58</v>
+        <v>924</v>
       </c>
       <c r="AK366" s="6">
-        <v>46301.927933530096</v>
+        <v>46296.93825494213</v>
       </c>
       <c r="AL366" s="3" t="s">
         <v>46</v>
@@ -49048,10 +49048,10 @@
         <v>46</v>
       </c>
       <c r="AN366" s="3" t="s">
-        <v>58</v>
+        <v>924</v>
       </c>
       <c r="AO366" s="6">
-        <v>46301.927933530096</v>
+        <v>46296.93825494213</v>
       </c>
     </row>
     <row r="367" spans="1:41" x14ac:dyDescent="0.25">
@@ -49080,28 +49080,28 @@
         <v>45</v>
       </c>
       <c r="I367" s="3" t="s">
-        <v>292</v>
+        <v>464</v>
       </c>
       <c r="J367" s="3" t="s">
-        <v>293</v>
+        <v>465</v>
       </c>
       <c r="K367" s="3" t="s">
-        <v>294</v>
+        <v>466</v>
       </c>
       <c r="L367" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M367" s="3" t="s">
-        <v>62</v>
+        <v>125</v>
       </c>
       <c r="N367" s="3" t="s">
-        <v>63</v>
+        <v>126</v>
       </c>
       <c r="O367" s="3" t="s">
-        <v>64</v>
+        <v>127</v>
       </c>
       <c r="P367" s="3" t="s">
-        <v>65</v>
+        <v>128</v>
       </c>
       <c r="Q367" s="5">
         <v>2</v>
@@ -49134,7 +49134,7 @@
         <v>46</v>
       </c>
       <c r="AA367" s="7">
-        <v>87000</v>
+        <v>1156433</v>
       </c>
       <c r="AB367" s="7">
         <v>1</v>
@@ -49205,28 +49205,28 @@
         <v>45</v>
       </c>
       <c r="I368" s="3" t="s">
-        <v>728</v>
+        <v>473</v>
       </c>
       <c r="J368" s="3" t="s">
-        <v>729</v>
+        <v>474</v>
       </c>
       <c r="K368" s="3" t="s">
-        <v>730</v>
+        <v>475</v>
       </c>
       <c r="L368" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M368" s="3" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="N368" s="3" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="O368" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="P368" s="3" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="Q368" s="5">
         <v>2</v>
@@ -49259,7 +49259,7 @@
         <v>46</v>
       </c>
       <c r="AA368" s="7">
-        <v>1567312</v>
+        <v>839166</v>
       </c>
       <c r="AB368" s="7">
         <v>1</v>
@@ -49330,28 +49330,28 @@
         <v>45</v>
       </c>
       <c r="I369" s="3" t="s">
-        <v>929</v>
+        <v>961</v>
       </c>
       <c r="J369" s="3" t="s">
-        <v>930</v>
+        <v>962</v>
       </c>
       <c r="K369" s="3" t="s">
-        <v>931</v>
+        <v>963</v>
       </c>
       <c r="L369" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M369" s="3" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="N369" s="3" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="O369" s="3" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="P369" s="3" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="Q369" s="5">
         <v>2</v>
@@ -49384,7 +49384,7 @@
         <v>46</v>
       </c>
       <c r="AA369" s="7">
-        <v>3025200</v>
+        <v>771000</v>
       </c>
       <c r="AB369" s="7">
         <v>1</v>
@@ -49461,31 +49461,31 @@
         <v>965</v>
       </c>
       <c r="K370" s="3" t="s">
-        <v>813</v>
+        <v>966</v>
       </c>
       <c r="L370" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M370" s="3" t="s">
-        <v>131</v>
+        <v>105</v>
       </c>
       <c r="N370" s="3" t="s">
-        <v>132</v>
+        <v>106</v>
       </c>
       <c r="O370" s="3" t="s">
-        <v>133</v>
+        <v>107</v>
       </c>
       <c r="P370" s="3" t="s">
-        <v>134</v>
+        <v>108</v>
       </c>
       <c r="Q370" s="5">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="R370" s="5">
         <v>2</v>
       </c>
       <c r="S370" s="5">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="T370" s="3" t="s">
         <v>894</v>
@@ -49509,7 +49509,7 @@
         <v>46</v>
       </c>
       <c r="AA370" s="7">
-        <v>468000</v>
+        <v>744240</v>
       </c>
       <c r="AB370" s="7">
         <v>1</v>
@@ -49580,13 +49580,13 @@
         <v>45</v>
       </c>
       <c r="I371" s="3" t="s">
-        <v>322</v>
+        <v>925</v>
       </c>
       <c r="J371" s="3" t="s">
-        <v>323</v>
+        <v>926</v>
       </c>
       <c r="K371" s="3" t="s">
-        <v>324</v>
+        <v>927</v>
       </c>
       <c r="L371" s="3" t="s">
         <v>50</v>
@@ -49633,8 +49633,8 @@
       <c r="Z371" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="AA371" s="7">
-        <v>5131620</v>
+      <c r="AA371" s="3" t="s">
+        <v>46</v>
       </c>
       <c r="AB371" s="7">
         <v>1</v>
@@ -49705,37 +49705,37 @@
         <v>45</v>
       </c>
       <c r="I372" s="3" t="s">
-        <v>740</v>
+        <v>393</v>
       </c>
       <c r="J372" s="3" t="s">
-        <v>741</v>
+        <v>394</v>
       </c>
       <c r="K372" s="3" t="s">
-        <v>742</v>
+        <v>395</v>
       </c>
       <c r="L372" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M372" s="3" t="s">
-        <v>69</v>
+        <v>105</v>
       </c>
       <c r="N372" s="3" t="s">
-        <v>70</v>
+        <v>106</v>
       </c>
       <c r="O372" s="3" t="s">
-        <v>71</v>
+        <v>107</v>
       </c>
       <c r="P372" s="3" t="s">
-        <v>72</v>
+        <v>108</v>
       </c>
       <c r="Q372" s="5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R372" s="5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S372" s="5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T372" s="3" t="s">
         <v>894</v>
@@ -49759,7 +49759,7 @@
         <v>46</v>
       </c>
       <c r="AA372" s="7">
-        <v>87000</v>
+        <v>692000</v>
       </c>
       <c r="AB372" s="7">
         <v>1</v>
@@ -49786,10 +49786,10 @@
         <v>0</v>
       </c>
       <c r="AJ372" s="3" t="s">
-        <v>924</v>
+        <v>58</v>
       </c>
       <c r="AK372" s="6">
-        <v>46296.93825494213</v>
+        <v>46302.79881820602</v>
       </c>
       <c r="AL372" s="3" t="s">
         <v>46</v>
@@ -49798,10 +49798,10 @@
         <v>46</v>
       </c>
       <c r="AN372" s="3" t="s">
-        <v>924</v>
+        <v>58</v>
       </c>
       <c r="AO372" s="6">
-        <v>46296.93825494213</v>
+        <v>46302.79881820602</v>
       </c>
     </row>
     <row r="373" spans="1:41" x14ac:dyDescent="0.25">
@@ -49955,37 +49955,37 @@
         <v>45</v>
       </c>
       <c r="I374" s="3" t="s">
-        <v>393</v>
+        <v>740</v>
       </c>
       <c r="J374" s="3" t="s">
-        <v>394</v>
+        <v>741</v>
       </c>
       <c r="K374" s="3" t="s">
-        <v>395</v>
+        <v>742</v>
       </c>
       <c r="L374" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M374" s="3" t="s">
-        <v>105</v>
+        <v>69</v>
       </c>
       <c r="N374" s="3" t="s">
-        <v>106</v>
+        <v>70</v>
       </c>
       <c r="O374" s="3" t="s">
-        <v>107</v>
+        <v>71</v>
       </c>
       <c r="P374" s="3" t="s">
-        <v>108</v>
+        <v>72</v>
       </c>
       <c r="Q374" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R374" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S374" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="T374" s="3" t="s">
         <v>894</v>
@@ -50009,7 +50009,7 @@
         <v>46</v>
       </c>
       <c r="AA374" s="7">
-        <v>692000</v>
+        <v>87000</v>
       </c>
       <c r="AB374" s="7">
         <v>1</v>
@@ -50036,10 +50036,10 @@
         <v>0</v>
       </c>
       <c r="AJ374" s="3" t="s">
-        <v>58</v>
+        <v>924</v>
       </c>
       <c r="AK374" s="6">
-        <v>46302.79881820602</v>
+        <v>46296.93825494213</v>
       </c>
       <c r="AL374" s="3" t="s">
         <v>46</v>
@@ -50048,10 +50048,10 @@
         <v>46</v>
       </c>
       <c r="AN374" s="3" t="s">
-        <v>58</v>
+        <v>924</v>
       </c>
       <c r="AO374" s="6">
-        <v>46302.79881820602</v>
+        <v>46296.93825494213</v>
       </c>
     </row>
     <row r="375" spans="1:41" x14ac:dyDescent="0.25">
@@ -50080,37 +50080,37 @@
         <v>45</v>
       </c>
       <c r="I375" s="3" t="s">
-        <v>925</v>
+        <v>967</v>
       </c>
       <c r="J375" s="3" t="s">
-        <v>926</v>
+        <v>968</v>
       </c>
       <c r="K375" s="3" t="s">
-        <v>927</v>
+        <v>813</v>
       </c>
       <c r="L375" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M375" s="3" t="s">
-        <v>105</v>
+        <v>131</v>
       </c>
       <c r="N375" s="3" t="s">
-        <v>106</v>
+        <v>132</v>
       </c>
       <c r="O375" s="3" t="s">
-        <v>107</v>
+        <v>133</v>
       </c>
       <c r="P375" s="3" t="s">
-        <v>108</v>
+        <v>134</v>
       </c>
       <c r="Q375" s="5">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="R375" s="5">
         <v>2</v>
       </c>
       <c r="S375" s="5">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="T375" s="3" t="s">
         <v>894</v>
@@ -50133,8 +50133,8 @@
       <c r="Z375" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="AA375" s="3" t="s">
-        <v>46</v>
+      <c r="AA375" s="7">
+        <v>468000</v>
       </c>
       <c r="AB375" s="7">
         <v>1</v>
@@ -50205,28 +50205,28 @@
         <v>45</v>
       </c>
       <c r="I376" s="3" t="s">
-        <v>966</v>
+        <v>929</v>
       </c>
       <c r="J376" s="3" t="s">
-        <v>967</v>
+        <v>930</v>
       </c>
       <c r="K376" s="3" t="s">
-        <v>968</v>
+        <v>931</v>
       </c>
       <c r="L376" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M376" s="3" t="s">
-        <v>105</v>
+        <v>125</v>
       </c>
       <c r="N376" s="3" t="s">
-        <v>106</v>
+        <v>126</v>
       </c>
       <c r="O376" s="3" t="s">
-        <v>107</v>
+        <v>127</v>
       </c>
       <c r="P376" s="3" t="s">
-        <v>108</v>
+        <v>128</v>
       </c>
       <c r="Q376" s="5">
         <v>2</v>
@@ -50259,7 +50259,7 @@
         <v>46</v>
       </c>
       <c r="AA376" s="7">
-        <v>744240</v>
+        <v>3025200</v>
       </c>
       <c r="AB376" s="7">
         <v>1</v>
@@ -50330,28 +50330,28 @@
         <v>45</v>
       </c>
       <c r="I377" s="3" t="s">
-        <v>969</v>
+        <v>722</v>
       </c>
       <c r="J377" s="3" t="s">
-        <v>970</v>
+        <v>723</v>
       </c>
       <c r="K377" s="3" t="s">
-        <v>971</v>
+        <v>724</v>
       </c>
       <c r="L377" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M377" s="3" t="s">
-        <v>131</v>
+        <v>62</v>
       </c>
       <c r="N377" s="3" t="s">
-        <v>132</v>
+        <v>63</v>
       </c>
       <c r="O377" s="3" t="s">
-        <v>133</v>
+        <v>64</v>
       </c>
       <c r="P377" s="3" t="s">
-        <v>134</v>
+        <v>65</v>
       </c>
       <c r="Q377" s="5">
         <v>2</v>
@@ -50384,7 +50384,7 @@
         <v>46</v>
       </c>
       <c r="AA377" s="7">
-        <v>771000</v>
+        <v>1227480</v>
       </c>
       <c r="AB377" s="7">
         <v>1</v>
@@ -50455,28 +50455,28 @@
         <v>45</v>
       </c>
       <c r="I378" s="3" t="s">
-        <v>422</v>
+        <v>144</v>
       </c>
       <c r="J378" s="3" t="s">
-        <v>423</v>
+        <v>145</v>
       </c>
       <c r="K378" s="3" t="s">
-        <v>424</v>
+        <v>146</v>
       </c>
       <c r="L378" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M378" s="3" t="s">
-        <v>131</v>
+        <v>98</v>
       </c>
       <c r="N378" s="3" t="s">
-        <v>132</v>
+        <v>99</v>
       </c>
       <c r="O378" s="3" t="s">
-        <v>133</v>
+        <v>100</v>
       </c>
       <c r="P378" s="3" t="s">
-        <v>134</v>
+        <v>101</v>
       </c>
       <c r="Q378" s="5">
         <v>2</v>
@@ -50509,7 +50509,7 @@
         <v>46</v>
       </c>
       <c r="AA378" s="7">
-        <v>698000</v>
+        <v>2736757</v>
       </c>
       <c r="AB378" s="7">
         <v>1</v>
@@ -50580,28 +50580,28 @@
         <v>45</v>
       </c>
       <c r="I379" s="3" t="s">
-        <v>772</v>
+        <v>135</v>
       </c>
       <c r="J379" s="3" t="s">
-        <v>773</v>
+        <v>136</v>
       </c>
       <c r="K379" s="3" t="s">
-        <v>774</v>
+        <v>137</v>
       </c>
       <c r="L379" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M379" s="3" t="s">
-        <v>62</v>
+        <v>131</v>
       </c>
       <c r="N379" s="3" t="s">
-        <v>63</v>
+        <v>132</v>
       </c>
       <c r="O379" s="3" t="s">
-        <v>64</v>
+        <v>133</v>
       </c>
       <c r="P379" s="3" t="s">
-        <v>65</v>
+        <v>134</v>
       </c>
       <c r="Q379" s="5">
         <v>2</v>
@@ -50634,7 +50634,7 @@
         <v>46</v>
       </c>
       <c r="AA379" s="7">
-        <v>2482921</v>
+        <v>536250</v>
       </c>
       <c r="AB379" s="7">
         <v>1</v>
@@ -50705,28 +50705,28 @@
         <v>45</v>
       </c>
       <c r="I380" s="3" t="s">
-        <v>464</v>
+        <v>109</v>
       </c>
       <c r="J380" s="3" t="s">
-        <v>465</v>
+        <v>110</v>
       </c>
       <c r="K380" s="3" t="s">
-        <v>466</v>
+        <v>111</v>
       </c>
       <c r="L380" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M380" s="3" t="s">
-        <v>125</v>
+        <v>62</v>
       </c>
       <c r="N380" s="3" t="s">
-        <v>126</v>
+        <v>63</v>
       </c>
       <c r="O380" s="3" t="s">
-        <v>127</v>
+        <v>64</v>
       </c>
       <c r="P380" s="3" t="s">
-        <v>128</v>
+        <v>65</v>
       </c>
       <c r="Q380" s="5">
         <v>2</v>
@@ -50759,7 +50759,7 @@
         <v>46</v>
       </c>
       <c r="AA380" s="7">
-        <v>1156433</v>
+        <v>558000</v>
       </c>
       <c r="AB380" s="7">
         <v>1</v>
@@ -50830,34 +50830,34 @@
         <v>45</v>
       </c>
       <c r="I381" s="3" t="s">
-        <v>473</v>
+        <v>969</v>
       </c>
       <c r="J381" s="3" t="s">
-        <v>474</v>
+        <v>970</v>
       </c>
       <c r="K381" s="3" t="s">
-        <v>475</v>
+        <v>971</v>
       </c>
       <c r="L381" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M381" s="3" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="N381" s="3" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="O381" s="3" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="P381" s="3" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="Q381" s="5">
         <v>2</v>
       </c>
       <c r="R381" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S381" s="5">
         <v>2</v>
@@ -50884,7 +50884,7 @@
         <v>46</v>
       </c>
       <c r="AA381" s="7">
-        <v>839166</v>
+        <v>646676</v>
       </c>
       <c r="AB381" s="7">
         <v>1</v>
@@ -50967,16 +50967,16 @@
         <v>50</v>
       </c>
       <c r="M382" s="3" t="s">
-        <v>105</v>
+        <v>125</v>
       </c>
       <c r="N382" s="3" t="s">
-        <v>106</v>
+        <v>126</v>
       </c>
       <c r="O382" s="3" t="s">
-        <v>107</v>
+        <v>127</v>
       </c>
       <c r="P382" s="3" t="s">
-        <v>108</v>
+        <v>128</v>
       </c>
       <c r="Q382" s="5">
         <v>2</v>
@@ -51009,7 +51009,7 @@
         <v>46</v>
       </c>
       <c r="AA382" s="7">
-        <v>384000</v>
+        <v>362000</v>
       </c>
       <c r="AB382" s="7">
         <v>1</v>
@@ -51217,16 +51217,16 @@
         <v>50</v>
       </c>
       <c r="M384" s="3" t="s">
-        <v>125</v>
+        <v>105</v>
       </c>
       <c r="N384" s="3" t="s">
-        <v>126</v>
+        <v>106</v>
       </c>
       <c r="O384" s="3" t="s">
-        <v>127</v>
+        <v>107</v>
       </c>
       <c r="P384" s="3" t="s">
-        <v>128</v>
+        <v>108</v>
       </c>
       <c r="Q384" s="5">
         <v>2</v>
@@ -51259,7 +51259,7 @@
         <v>46</v>
       </c>
       <c r="AA384" s="7">
-        <v>362000</v>
+        <v>384000</v>
       </c>
       <c r="AB384" s="7">
         <v>1</v>
@@ -52455,13 +52455,13 @@
         <v>45</v>
       </c>
       <c r="I394" s="3" t="s">
-        <v>912</v>
+        <v>909</v>
       </c>
       <c r="J394" s="3" t="s">
-        <v>913</v>
+        <v>910</v>
       </c>
       <c r="K394" s="3" t="s">
-        <v>914</v>
+        <v>911</v>
       </c>
       <c r="L394" s="3" t="s">
         <v>50</v>
@@ -53205,13 +53205,13 @@
         <v>45</v>
       </c>
       <c r="I400" s="3" t="s">
-        <v>900</v>
+        <v>915</v>
       </c>
       <c r="J400" s="3" t="s">
-        <v>901</v>
+        <v>916</v>
       </c>
       <c r="K400" s="3" t="s">
-        <v>902</v>
+        <v>917</v>
       </c>
       <c r="L400" s="3" t="s">
         <v>50</v>
@@ -53729,13 +53729,13 @@
         <v>128</v>
       </c>
       <c r="Q404" s="5">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="R404" s="5">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="S404" s="5">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="T404" s="3" t="s">
         <v>894</v>
@@ -55205,10 +55205,10 @@
         <v>999</v>
       </c>
       <c r="I416" s="3" t="s">
-        <v>964</v>
+        <v>967</v>
       </c>
       <c r="J416" s="3" t="s">
-        <v>965</v>
+        <v>968</v>
       </c>
       <c r="K416" s="3" t="s">
         <v>813</v>
@@ -57604,13 +57604,13 @@
         <v>156</v>
       </c>
       <c r="Q435" s="5">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="R435" s="5">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="S435" s="5">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="T435" s="3" t="s">
         <v>894</v>
@@ -58729,13 +58729,13 @@
         <v>134</v>
       </c>
       <c r="Q444" s="5">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="R444" s="5">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="S444" s="5">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="T444" s="3" t="s">
         <v>894</v>
@@ -60205,13 +60205,13 @@
         <v>921</v>
       </c>
       <c r="I456" s="3" t="s">
-        <v>900</v>
+        <v>915</v>
       </c>
       <c r="J456" s="3" t="s">
-        <v>901</v>
+        <v>916</v>
       </c>
       <c r="K456" s="3" t="s">
-        <v>902</v>
+        <v>917</v>
       </c>
       <c r="L456" s="3" t="s">
         <v>50</v>
@@ -60854,13 +60854,13 @@
         <v>128</v>
       </c>
       <c r="Q461" s="5">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="R461" s="5">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="S461" s="5">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="T461" s="3" t="s">
         <v>894</v>
@@ -61354,13 +61354,13 @@
         <v>156</v>
       </c>
       <c r="Q465" s="5">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="R465" s="5">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="S465" s="5">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="T465" s="3" t="s">
         <v>894</v>
@@ -61455,13 +61455,13 @@
         <v>45</v>
       </c>
       <c r="I466" s="3" t="s">
-        <v>955</v>
+        <v>969</v>
       </c>
       <c r="J466" s="3" t="s">
-        <v>956</v>
+        <v>970</v>
       </c>
       <c r="K466" s="3" t="s">
-        <v>957</v>
+        <v>971</v>
       </c>
       <c r="L466" s="3" t="s">
         <v>50</v>
@@ -61854,13 +61854,13 @@
         <v>156</v>
       </c>
       <c r="Q469" s="5">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="R469" s="5">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="S469" s="5">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="T469" s="3" t="s">
         <v>894</v>
@@ -62229,13 +62229,13 @@
         <v>156</v>
       </c>
       <c r="Q472" s="5">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="R472" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S472" s="5">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T472" s="3" t="s">
         <v>894</v>
@@ -62354,13 +62354,13 @@
         <v>156</v>
       </c>
       <c r="Q473" s="5">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="R473" s="5">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S473" s="5">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T473" s="3" t="s">
         <v>894</v>
@@ -62604,13 +62604,13 @@
         <v>156</v>
       </c>
       <c r="Q475" s="5">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="R475" s="5">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="S475" s="5">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="T475" s="3" t="s">
         <v>894</v>
@@ -62705,10 +62705,10 @@
         <v>45</v>
       </c>
       <c r="I476" s="3" t="s">
-        <v>964</v>
+        <v>967</v>
       </c>
       <c r="J476" s="3" t="s">
-        <v>965</v>
+        <v>968</v>
       </c>
       <c r="K476" s="3" t="s">
         <v>813</v>

</xml_diff>

<commit_message>
Auto sync Onetech 28/10/2026 17:53
</commit_message>
<xml_diff>
--- a/data/Thang10/DANH_SACH_KET_QUA_CUA_HANG_THAM_GIA_CHUONG_TRINH.xlsx
+++ b/data/Thang10/DANH_SACH_KET_QUA_CUA_HANG_THAM_GIA_CHUONG_TRINH.xlsx
@@ -2713,6 +2713,15 @@
     <t>Active</t>
   </si>
   <si>
+    <t>3362</t>
+  </si>
+  <si>
+    <t>Thủy Kết</t>
+  </si>
+  <si>
+    <t>107, Lò Lu</t>
+  </si>
+  <si>
     <t>999754600</t>
   </si>
   <si>
@@ -2758,15 +2767,6 @@
     <t>40 Cảng Phú Hữu, Nguyễn Duy Trinh</t>
   </si>
   <si>
-    <t>3362</t>
-  </si>
-  <si>
-    <t>Thủy Kết</t>
-  </si>
-  <si>
-    <t>107, Lò Lu</t>
-  </si>
-  <si>
     <t>1-6JP933U</t>
   </si>
   <si>
@@ -2878,6 +2878,15 @@
     <t>MSC_BEV_Chương trình TBTN_Tủ mát Nước giải khát_HCM_All2026_T10</t>
   </si>
   <si>
+    <t>2128924</t>
+  </si>
+  <si>
+    <t>Tạp Hoá Hồng Ngọc</t>
+  </si>
+  <si>
+    <t>22/10 Đường 990, Nguyễn Duy Trinh</t>
+  </si>
+  <si>
     <t>2432200</t>
   </si>
   <si>
@@ -2896,6 +2905,21 @@
     <t>242, Đường 57 - CL</t>
   </si>
   <si>
+    <t>2894640</t>
+  </si>
+  <si>
+    <t>Mino Mart</t>
+  </si>
+  <si>
+    <t>3063948</t>
+  </si>
+  <si>
+    <t>Cà Phê Chị Tuyết</t>
+  </si>
+  <si>
+    <t>Đối Diện Cổng E, Đường Số 57 CL</t>
+  </si>
+  <si>
     <t>3136368</t>
   </si>
   <si>
@@ -2905,28 +2929,13 @@
     <t>35 Đường Số 12, Bưng Ông Thoàn</t>
   </si>
   <si>
-    <t>3063948</t>
-  </si>
-  <si>
-    <t>Cà Phê Chị Tuyết</t>
-  </si>
-  <si>
-    <t>Đối Diện Cổng E, Đường Số 57 CL</t>
-  </si>
-  <si>
-    <t>2894640</t>
-  </si>
-  <si>
-    <t>Mino Mart</t>
-  </si>
-  <si>
-    <t>2128924</t>
-  </si>
-  <si>
-    <t>Tạp Hoá Hồng Ngọc</t>
-  </si>
-  <si>
-    <t>22/10 Đường 990, Nguyễn Duy Trinh</t>
+    <t>999115327</t>
+  </si>
+  <si>
+    <t>Hà Thủy</t>
+  </si>
+  <si>
+    <t>Số 313, Lê Văn Thịnh</t>
   </si>
   <si>
     <t>999191040</t>
@@ -2936,15 +2945,6 @@
   </si>
   <si>
     <t>250, Trường Lưu</t>
-  </si>
-  <si>
-    <t>999115327</t>
-  </si>
-  <si>
-    <t>Hà Thủy</t>
-  </si>
-  <si>
-    <t>Số 313, Lê Văn Thịnh</t>
   </si>
   <si>
     <t>999210374</t>
@@ -42092,16 +42092,16 @@
         <v>50</v>
       </c>
       <c r="M311" s="3" t="s">
-        <v>62</v>
+        <v>115</v>
       </c>
       <c r="N311" s="3" t="s">
-        <v>63</v>
+        <v>116</v>
       </c>
       <c r="O311" s="3" t="s">
-        <v>64</v>
+        <v>117</v>
       </c>
       <c r="P311" s="3" t="s">
-        <v>65</v>
+        <v>118</v>
       </c>
       <c r="Q311" s="3" t="s">
         <v>46</v>
@@ -42134,7 +42134,7 @@
         <v>10</v>
       </c>
       <c r="AA311" s="7">
-        <v>10.75</v>
+        <v>10</v>
       </c>
       <c r="AB311" s="7">
         <v>1</v>
@@ -42164,7 +42164,7 @@
         <v>58</v>
       </c>
       <c r="AK311" s="6">
-        <v>46312.58308098379</v>
+        <v>46298.66540524305</v>
       </c>
       <c r="AL311" s="3" t="s">
         <v>46</v>
@@ -42176,7 +42176,7 @@
         <v>58</v>
       </c>
       <c r="AO311" s="6">
-        <v>46312.58308098379</v>
+        <v>46298.66540524305</v>
       </c>
     </row>
     <row r="312" spans="1:41" x14ac:dyDescent="0.25">
@@ -42217,16 +42217,16 @@
         <v>50</v>
       </c>
       <c r="M312" s="3" t="s">
-        <v>105</v>
+        <v>62</v>
       </c>
       <c r="N312" s="3" t="s">
-        <v>106</v>
+        <v>63</v>
       </c>
       <c r="O312" s="3" t="s">
-        <v>107</v>
+        <v>64</v>
       </c>
       <c r="P312" s="3" t="s">
-        <v>108</v>
+        <v>65</v>
       </c>
       <c r="Q312" s="3" t="s">
         <v>46</v>
@@ -42259,7 +42259,7 @@
         <v>10</v>
       </c>
       <c r="AA312" s="7">
-        <v>10</v>
+        <v>10.75</v>
       </c>
       <c r="AB312" s="7">
         <v>1</v>
@@ -42289,7 +42289,7 @@
         <v>58</v>
       </c>
       <c r="AK312" s="6">
-        <v>46310.439036655094</v>
+        <v>46312.58308098379</v>
       </c>
       <c r="AL312" s="3" t="s">
         <v>46</v>
@@ -42301,7 +42301,7 @@
         <v>58</v>
       </c>
       <c r="AO312" s="6">
-        <v>46310.439036655094</v>
+        <v>46312.58308098379</v>
       </c>
     </row>
     <row r="313" spans="1:41" x14ac:dyDescent="0.25">
@@ -42342,16 +42342,16 @@
         <v>50</v>
       </c>
       <c r="M313" s="3" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="N313" s="3" t="s">
-        <v>116</v>
+        <v>106</v>
       </c>
       <c r="O313" s="3" t="s">
-        <v>117</v>
+        <v>107</v>
       </c>
       <c r="P313" s="3" t="s">
-        <v>118</v>
+        <v>108</v>
       </c>
       <c r="Q313" s="3" t="s">
         <v>46</v>
@@ -42414,7 +42414,7 @@
         <v>58</v>
       </c>
       <c r="AK313" s="6">
-        <v>46301.30899568287</v>
+        <v>46310.439036655094</v>
       </c>
       <c r="AL313" s="3" t="s">
         <v>46</v>
@@ -42426,7 +42426,7 @@
         <v>58</v>
       </c>
       <c r="AO313" s="6">
-        <v>46301.30899568287</v>
+        <v>46310.439036655094</v>
       </c>
     </row>
     <row r="314" spans="1:41" x14ac:dyDescent="0.25">
@@ -42455,28 +42455,28 @@
         <v>45</v>
       </c>
       <c r="I314" s="3" t="s">
-        <v>271</v>
+        <v>909</v>
       </c>
       <c r="J314" s="3" t="s">
-        <v>272</v>
+        <v>910</v>
       </c>
       <c r="K314" s="3" t="s">
-        <v>273</v>
+        <v>911</v>
       </c>
       <c r="L314" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M314" s="3" t="s">
-        <v>79</v>
+        <v>115</v>
       </c>
       <c r="N314" s="3" t="s">
-        <v>80</v>
+        <v>116</v>
       </c>
       <c r="O314" s="3" t="s">
-        <v>81</v>
+        <v>117</v>
       </c>
       <c r="P314" s="3" t="s">
-        <v>82</v>
+        <v>118</v>
       </c>
       <c r="Q314" s="3" t="s">
         <v>46</v>
@@ -42539,7 +42539,7 @@
         <v>58</v>
       </c>
       <c r="AK314" s="6">
-        <v>46301.5776272338</v>
+        <v>46301.30899568287</v>
       </c>
       <c r="AL314" s="3" t="s">
         <v>46</v>
@@ -42551,7 +42551,7 @@
         <v>58</v>
       </c>
       <c r="AO314" s="6">
-        <v>46301.5776272338</v>
+        <v>46301.30899568287</v>
       </c>
     </row>
     <row r="315" spans="1:41" x14ac:dyDescent="0.25">
@@ -42580,28 +42580,28 @@
         <v>45</v>
       </c>
       <c r="I315" s="3" t="s">
-        <v>322</v>
+        <v>271</v>
       </c>
       <c r="J315" s="3" t="s">
-        <v>323</v>
+        <v>272</v>
       </c>
       <c r="K315" s="3" t="s">
-        <v>324</v>
+        <v>273</v>
       </c>
       <c r="L315" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M315" s="3" t="s">
-        <v>105</v>
+        <v>79</v>
       </c>
       <c r="N315" s="3" t="s">
-        <v>106</v>
+        <v>80</v>
       </c>
       <c r="O315" s="3" t="s">
-        <v>107</v>
+        <v>81</v>
       </c>
       <c r="P315" s="3" t="s">
-        <v>108</v>
+        <v>82</v>
       </c>
       <c r="Q315" s="3" t="s">
         <v>46</v>
@@ -42634,7 +42634,7 @@
         <v>10</v>
       </c>
       <c r="AA315" s="7">
-        <v>10.5</v>
+        <v>10</v>
       </c>
       <c r="AB315" s="7">
         <v>1</v>
@@ -42664,7 +42664,7 @@
         <v>58</v>
       </c>
       <c r="AK315" s="6">
-        <v>46303.59483915509</v>
+        <v>46301.5776272338</v>
       </c>
       <c r="AL315" s="3" t="s">
         <v>46</v>
@@ -42676,7 +42676,7 @@
         <v>58</v>
       </c>
       <c r="AO315" s="6">
-        <v>46303.59483915509</v>
+        <v>46301.5776272338</v>
       </c>
     </row>
     <row r="316" spans="1:41" x14ac:dyDescent="0.25">
@@ -42705,28 +42705,28 @@
         <v>45</v>
       </c>
       <c r="I316" s="3" t="s">
-        <v>150</v>
+        <v>322</v>
       </c>
       <c r="J316" s="3" t="s">
-        <v>151</v>
+        <v>323</v>
       </c>
       <c r="K316" s="3" t="s">
-        <v>152</v>
+        <v>324</v>
       </c>
       <c r="L316" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M316" s="3" t="s">
-        <v>153</v>
+        <v>105</v>
       </c>
       <c r="N316" s="3" t="s">
-        <v>154</v>
+        <v>106</v>
       </c>
       <c r="O316" s="3" t="s">
-        <v>155</v>
+        <v>107</v>
       </c>
       <c r="P316" s="3" t="s">
-        <v>156</v>
+        <v>108</v>
       </c>
       <c r="Q316" s="3" t="s">
         <v>46</v>
@@ -42759,7 +42759,7 @@
         <v>10</v>
       </c>
       <c r="AA316" s="7">
-        <v>10</v>
+        <v>10.5</v>
       </c>
       <c r="AB316" s="7">
         <v>1</v>
@@ -42789,7 +42789,7 @@
         <v>58</v>
       </c>
       <c r="AK316" s="6">
-        <v>46298.66540524305</v>
+        <v>46303.59483915509</v>
       </c>
       <c r="AL316" s="3" t="s">
         <v>46</v>
@@ -42801,7 +42801,7 @@
         <v>58</v>
       </c>
       <c r="AO316" s="6">
-        <v>46298.66540524305</v>
+        <v>46303.59483915509</v>
       </c>
     </row>
     <row r="317" spans="1:41" x14ac:dyDescent="0.25">
@@ -42830,28 +42830,28 @@
         <v>45</v>
       </c>
       <c r="I317" s="3" t="s">
-        <v>909</v>
+        <v>150</v>
       </c>
       <c r="J317" s="3" t="s">
-        <v>910</v>
+        <v>151</v>
       </c>
       <c r="K317" s="3" t="s">
-        <v>911</v>
+        <v>152</v>
       </c>
       <c r="L317" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M317" s="3" t="s">
-        <v>115</v>
+        <v>153</v>
       </c>
       <c r="N317" s="3" t="s">
-        <v>116</v>
+        <v>154</v>
       </c>
       <c r="O317" s="3" t="s">
-        <v>117</v>
+        <v>155</v>
       </c>
       <c r="P317" s="3" t="s">
-        <v>118</v>
+        <v>156</v>
       </c>
       <c r="Q317" s="3" t="s">
         <v>46</v>
@@ -42967,16 +42967,16 @@
         <v>50</v>
       </c>
       <c r="M318" s="3" t="s">
-        <v>131</v>
+        <v>115</v>
       </c>
       <c r="N318" s="3" t="s">
-        <v>132</v>
+        <v>116</v>
       </c>
       <c r="O318" s="3" t="s">
-        <v>133</v>
+        <v>117</v>
       </c>
       <c r="P318" s="3" t="s">
-        <v>134</v>
+        <v>118</v>
       </c>
       <c r="Q318" s="3" t="s">
         <v>46</v>
@@ -43039,7 +43039,7 @@
         <v>58</v>
       </c>
       <c r="AK318" s="6">
-        <v>46316.79383703704</v>
+        <v>46298.66540524305</v>
       </c>
       <c r="AL318" s="3" t="s">
         <v>46</v>
@@ -43051,7 +43051,7 @@
         <v>58</v>
       </c>
       <c r="AO318" s="6">
-        <v>46316.79383703704</v>
+        <v>46298.66540524305</v>
       </c>
     </row>
     <row r="319" spans="1:41" x14ac:dyDescent="0.25">
@@ -43080,28 +43080,28 @@
         <v>45</v>
       </c>
       <c r="I319" s="3" t="s">
-        <v>138</v>
+        <v>915</v>
       </c>
       <c r="J319" s="3" t="s">
-        <v>139</v>
+        <v>916</v>
       </c>
       <c r="K319" s="3" t="s">
-        <v>140</v>
+        <v>917</v>
       </c>
       <c r="L319" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M319" s="3" t="s">
-        <v>105</v>
+        <v>131</v>
       </c>
       <c r="N319" s="3" t="s">
-        <v>106</v>
+        <v>132</v>
       </c>
       <c r="O319" s="3" t="s">
-        <v>107</v>
+        <v>133</v>
       </c>
       <c r="P319" s="3" t="s">
-        <v>108</v>
+        <v>134</v>
       </c>
       <c r="Q319" s="3" t="s">
         <v>46</v>
@@ -43134,7 +43134,7 @@
         <v>10</v>
       </c>
       <c r="AA319" s="7">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="AB319" s="7">
         <v>1</v>
@@ -43164,7 +43164,7 @@
         <v>58</v>
       </c>
       <c r="AK319" s="6">
-        <v>46303.59483915509</v>
+        <v>46316.79383703704</v>
       </c>
       <c r="AL319" s="3" t="s">
         <v>46</v>
@@ -43176,7 +43176,7 @@
         <v>58</v>
       </c>
       <c r="AO319" s="6">
-        <v>46303.59483915509</v>
+        <v>46316.79383703704</v>
       </c>
     </row>
     <row r="320" spans="1:41" x14ac:dyDescent="0.25">
@@ -43205,28 +43205,28 @@
         <v>45</v>
       </c>
       <c r="I320" s="3" t="s">
-        <v>915</v>
+        <v>138</v>
       </c>
       <c r="J320" s="3" t="s">
-        <v>916</v>
+        <v>139</v>
       </c>
       <c r="K320" s="3" t="s">
-        <v>917</v>
+        <v>140</v>
       </c>
       <c r="L320" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M320" s="3" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="N320" s="3" t="s">
-        <v>116</v>
+        <v>106</v>
       </c>
       <c r="O320" s="3" t="s">
-        <v>117</v>
+        <v>107</v>
       </c>
       <c r="P320" s="3" t="s">
-        <v>118</v>
+        <v>108</v>
       </c>
       <c r="Q320" s="3" t="s">
         <v>46</v>
@@ -43259,7 +43259,7 @@
         <v>10</v>
       </c>
       <c r="AA320" s="7">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="AB320" s="7">
         <v>1</v>
@@ -43289,7 +43289,7 @@
         <v>58</v>
       </c>
       <c r="AK320" s="6">
-        <v>46298.66540524305</v>
+        <v>46303.59483915509</v>
       </c>
       <c r="AL320" s="3" t="s">
         <v>46</v>
@@ -43301,7 +43301,7 @@
         <v>58</v>
       </c>
       <c r="AO320" s="6">
-        <v>46298.66540524305</v>
+        <v>46303.59483915509</v>
       </c>
     </row>
     <row r="321" spans="1:41" x14ac:dyDescent="0.25">
@@ -46455,37 +46455,37 @@
         <v>921</v>
       </c>
       <c r="I346" s="3" t="s">
-        <v>939</v>
+        <v>378</v>
       </c>
       <c r="J346" s="3" t="s">
-        <v>744</v>
+        <v>379</v>
       </c>
       <c r="K346" s="3" t="s">
-        <v>940</v>
+        <v>380</v>
       </c>
       <c r="L346" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M346" s="3" t="s">
-        <v>79</v>
+        <v>125</v>
       </c>
       <c r="N346" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="O346" s="3" t="s">
-        <v>81</v>
+        <v>127</v>
       </c>
       <c r="P346" s="3" t="s">
-        <v>82</v>
+        <v>128</v>
       </c>
       <c r="Q346" s="5">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="R346" s="5">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="S346" s="5">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="T346" s="3" t="s">
         <v>894</v>
@@ -46509,7 +46509,7 @@
         <v>46</v>
       </c>
       <c r="AA346" s="7">
-        <v>2416326</v>
+        <v>156000</v>
       </c>
       <c r="AB346" s="7">
         <v>31</v>
@@ -46580,37 +46580,37 @@
         <v>921</v>
       </c>
       <c r="I347" s="3" t="s">
-        <v>948</v>
+        <v>939</v>
       </c>
       <c r="J347" s="3" t="s">
-        <v>949</v>
+        <v>744</v>
       </c>
       <c r="K347" s="3" t="s">
-        <v>950</v>
+        <v>940</v>
       </c>
       <c r="L347" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M347" s="3" t="s">
-        <v>131</v>
+        <v>79</v>
       </c>
       <c r="N347" s="3" t="s">
-        <v>132</v>
+        <v>80</v>
       </c>
       <c r="O347" s="3" t="s">
-        <v>133</v>
+        <v>81</v>
       </c>
       <c r="P347" s="3" t="s">
-        <v>134</v>
+        <v>82</v>
       </c>
       <c r="Q347" s="5">
-        <v>26</v>
+        <v>7</v>
       </c>
       <c r="R347" s="5">
-        <v>26</v>
+        <v>3</v>
       </c>
       <c r="S347" s="5">
-        <v>26</v>
+        <v>7</v>
       </c>
       <c r="T347" s="3" t="s">
         <v>894</v>
@@ -46634,7 +46634,7 @@
         <v>46</v>
       </c>
       <c r="AA347" s="7">
-        <v>2359523</v>
+        <v>2416326</v>
       </c>
       <c r="AB347" s="7">
         <v>31</v>
@@ -46705,37 +46705,37 @@
         <v>921</v>
       </c>
       <c r="I348" s="3" t="s">
-        <v>755</v>
+        <v>948</v>
       </c>
       <c r="J348" s="3" t="s">
-        <v>756</v>
+        <v>949</v>
       </c>
       <c r="K348" s="3" t="s">
-        <v>757</v>
+        <v>950</v>
       </c>
       <c r="L348" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M348" s="3" t="s">
-        <v>115</v>
+        <v>131</v>
       </c>
       <c r="N348" s="3" t="s">
-        <v>116</v>
+        <v>132</v>
       </c>
       <c r="O348" s="3" t="s">
-        <v>117</v>
+        <v>133</v>
       </c>
       <c r="P348" s="3" t="s">
-        <v>118</v>
+        <v>134</v>
       </c>
       <c r="Q348" s="5">
-        <v>13</v>
+        <v>26</v>
       </c>
       <c r="R348" s="5">
-        <v>13</v>
+        <v>26</v>
       </c>
       <c r="S348" s="5">
-        <v>13</v>
+        <v>26</v>
       </c>
       <c r="T348" s="3" t="s">
         <v>894</v>
@@ -46759,7 +46759,7 @@
         <v>46</v>
       </c>
       <c r="AA348" s="7">
-        <v>2580460</v>
+        <v>2359523</v>
       </c>
       <c r="AB348" s="7">
         <v>31</v>
@@ -46830,37 +46830,37 @@
         <v>921</v>
       </c>
       <c r="I349" s="3" t="s">
-        <v>464</v>
+        <v>755</v>
       </c>
       <c r="J349" s="3" t="s">
-        <v>465</v>
+        <v>756</v>
       </c>
       <c r="K349" s="3" t="s">
-        <v>466</v>
+        <v>757</v>
       </c>
       <c r="L349" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M349" s="3" t="s">
-        <v>125</v>
+        <v>115</v>
       </c>
       <c r="N349" s="3" t="s">
-        <v>126</v>
+        <v>116</v>
       </c>
       <c r="O349" s="3" t="s">
-        <v>127</v>
+        <v>117</v>
       </c>
       <c r="P349" s="3" t="s">
-        <v>128</v>
+        <v>118</v>
       </c>
       <c r="Q349" s="5">
-        <v>34</v>
+        <v>13</v>
       </c>
       <c r="R349" s="5">
-        <v>34</v>
+        <v>13</v>
       </c>
       <c r="S349" s="5">
-        <v>34</v>
+        <v>13</v>
       </c>
       <c r="T349" s="3" t="s">
         <v>894</v>
@@ -46884,7 +46884,7 @@
         <v>46</v>
       </c>
       <c r="AA349" s="7">
-        <v>570000</v>
+        <v>2580460</v>
       </c>
       <c r="AB349" s="7">
         <v>31</v>
@@ -46955,13 +46955,13 @@
         <v>921</v>
       </c>
       <c r="I350" s="3" t="s">
-        <v>473</v>
+        <v>464</v>
       </c>
       <c r="J350" s="3" t="s">
-        <v>474</v>
+        <v>465</v>
       </c>
       <c r="K350" s="3" t="s">
-        <v>475</v>
+        <v>466</v>
       </c>
       <c r="L350" s="3" t="s">
         <v>50</v>
@@ -46979,13 +46979,13 @@
         <v>128</v>
       </c>
       <c r="Q350" s="5">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="R350" s="5">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="S350" s="5">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="T350" s="3" t="s">
         <v>894</v>
@@ -47009,7 +47009,7 @@
         <v>46</v>
       </c>
       <c r="AA350" s="7">
-        <v>925650</v>
+        <v>570000</v>
       </c>
       <c r="AB350" s="7">
         <v>31</v>
@@ -47080,13 +47080,13 @@
         <v>921</v>
       </c>
       <c r="I351" s="3" t="s">
-        <v>535</v>
+        <v>473</v>
       </c>
       <c r="J351" s="3" t="s">
-        <v>536</v>
+        <v>474</v>
       </c>
       <c r="K351" s="3" t="s">
-        <v>537</v>
+        <v>475</v>
       </c>
       <c r="L351" s="3" t="s">
         <v>50</v>
@@ -47104,13 +47104,13 @@
         <v>128</v>
       </c>
       <c r="Q351" s="5">
-        <v>5</v>
+        <v>28</v>
       </c>
       <c r="R351" s="5">
-        <v>3</v>
+        <v>28</v>
       </c>
       <c r="S351" s="5">
-        <v>6</v>
+        <v>28</v>
       </c>
       <c r="T351" s="3" t="s">
         <v>894</v>
@@ -47134,7 +47134,7 @@
         <v>46</v>
       </c>
       <c r="AA351" s="7">
-        <v>590000</v>
+        <v>925650</v>
       </c>
       <c r="AB351" s="7">
         <v>31</v>
@@ -47205,13 +47205,13 @@
         <v>921</v>
       </c>
       <c r="I352" s="3" t="s">
-        <v>575</v>
+        <v>535</v>
       </c>
       <c r="J352" s="3" t="s">
-        <v>576</v>
+        <v>536</v>
       </c>
       <c r="K352" s="3" t="s">
-        <v>577</v>
+        <v>537</v>
       </c>
       <c r="L352" s="3" t="s">
         <v>50</v>
@@ -47229,13 +47229,13 @@
         <v>128</v>
       </c>
       <c r="Q352" s="5">
-        <v>27</v>
+        <v>5</v>
       </c>
       <c r="R352" s="5">
-        <v>26</v>
+        <v>3</v>
       </c>
       <c r="S352" s="5">
-        <v>28</v>
+        <v>6</v>
       </c>
       <c r="T352" s="3" t="s">
         <v>894</v>
@@ -47259,7 +47259,7 @@
         <v>46</v>
       </c>
       <c r="AA352" s="7">
-        <v>2566500</v>
+        <v>590000</v>
       </c>
       <c r="AB352" s="7">
         <v>31</v>
@@ -47330,13 +47330,13 @@
         <v>921</v>
       </c>
       <c r="I353" s="3" t="s">
-        <v>578</v>
+        <v>575</v>
       </c>
       <c r="J353" s="3" t="s">
-        <v>579</v>
+        <v>576</v>
       </c>
       <c r="K353" s="3" t="s">
-        <v>580</v>
+        <v>577</v>
       </c>
       <c r="L353" s="3" t="s">
         <v>50</v>
@@ -47354,13 +47354,13 @@
         <v>128</v>
       </c>
       <c r="Q353" s="5">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="R353" s="5">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="S353" s="5">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="T353" s="3" t="s">
         <v>894</v>
@@ -47383,8 +47383,8 @@
       <c r="Z353" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="AA353" s="3" t="s">
-        <v>46</v>
+      <c r="AA353" s="7">
+        <v>2566500</v>
       </c>
       <c r="AB353" s="7">
         <v>31</v>
@@ -47455,37 +47455,37 @@
         <v>921</v>
       </c>
       <c r="I354" s="3" t="s">
-        <v>89</v>
+        <v>578</v>
       </c>
       <c r="J354" s="3" t="s">
-        <v>90</v>
+        <v>579</v>
       </c>
       <c r="K354" s="3" t="s">
-        <v>91</v>
+        <v>580</v>
       </c>
       <c r="L354" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M354" s="3" t="s">
-        <v>69</v>
+        <v>125</v>
       </c>
       <c r="N354" s="3" t="s">
-        <v>70</v>
+        <v>126</v>
       </c>
       <c r="O354" s="3" t="s">
-        <v>71</v>
+        <v>127</v>
       </c>
       <c r="P354" s="3" t="s">
-        <v>72</v>
+        <v>128</v>
       </c>
       <c r="Q354" s="5">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="R354" s="5">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="S354" s="5">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="T354" s="3" t="s">
         <v>894</v>
@@ -47508,8 +47508,8 @@
       <c r="Z354" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="AA354" s="7">
-        <v>1246838</v>
+      <c r="AA354" s="3" t="s">
+        <v>46</v>
       </c>
       <c r="AB354" s="7">
         <v>31</v>
@@ -47580,37 +47580,37 @@
         <v>921</v>
       </c>
       <c r="I355" s="3" t="s">
-        <v>699</v>
+        <v>659</v>
       </c>
       <c r="J355" s="3" t="s">
-        <v>700</v>
+        <v>660</v>
       </c>
       <c r="K355" s="3" t="s">
-        <v>701</v>
+        <v>661</v>
       </c>
       <c r="L355" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M355" s="3" t="s">
-        <v>115</v>
+        <v>125</v>
       </c>
       <c r="N355" s="3" t="s">
-        <v>116</v>
+        <v>126</v>
       </c>
       <c r="O355" s="3" t="s">
-        <v>117</v>
+        <v>127</v>
       </c>
       <c r="P355" s="3" t="s">
-        <v>118</v>
+        <v>128</v>
       </c>
       <c r="Q355" s="5">
-        <v>35</v>
+        <v>26</v>
       </c>
       <c r="R355" s="5">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="S355" s="5">
-        <v>35</v>
+        <v>26</v>
       </c>
       <c r="T355" s="3" t="s">
         <v>894</v>
@@ -47634,7 +47634,7 @@
         <v>46</v>
       </c>
       <c r="AA355" s="7">
-        <v>339000</v>
+        <v>290939</v>
       </c>
       <c r="AB355" s="7">
         <v>31</v>
@@ -47705,37 +47705,37 @@
         <v>921</v>
       </c>
       <c r="I356" s="3" t="s">
-        <v>659</v>
+        <v>89</v>
       </c>
       <c r="J356" s="3" t="s">
-        <v>660</v>
+        <v>90</v>
       </c>
       <c r="K356" s="3" t="s">
-        <v>661</v>
+        <v>91</v>
       </c>
       <c r="L356" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M356" s="3" t="s">
-        <v>125</v>
+        <v>69</v>
       </c>
       <c r="N356" s="3" t="s">
-        <v>126</v>
+        <v>70</v>
       </c>
       <c r="O356" s="3" t="s">
-        <v>127</v>
+        <v>71</v>
       </c>
       <c r="P356" s="3" t="s">
-        <v>128</v>
+        <v>72</v>
       </c>
       <c r="Q356" s="5">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="R356" s="5">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="S356" s="5">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="T356" s="3" t="s">
         <v>894</v>
@@ -47759,7 +47759,7 @@
         <v>46</v>
       </c>
       <c r="AA356" s="7">
-        <v>290939</v>
+        <v>1246838</v>
       </c>
       <c r="AB356" s="7">
         <v>31</v>
@@ -47830,37 +47830,37 @@
         <v>921</v>
       </c>
       <c r="I357" s="3" t="s">
-        <v>378</v>
+        <v>699</v>
       </c>
       <c r="J357" s="3" t="s">
-        <v>379</v>
+        <v>700</v>
       </c>
       <c r="K357" s="3" t="s">
-        <v>380</v>
+        <v>701</v>
       </c>
       <c r="L357" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M357" s="3" t="s">
-        <v>125</v>
+        <v>115</v>
       </c>
       <c r="N357" s="3" t="s">
-        <v>126</v>
+        <v>116</v>
       </c>
       <c r="O357" s="3" t="s">
-        <v>127</v>
+        <v>117</v>
       </c>
       <c r="P357" s="3" t="s">
-        <v>128</v>
+        <v>118</v>
       </c>
       <c r="Q357" s="5">
-        <v>10</v>
+        <v>35</v>
       </c>
       <c r="R357" s="5">
-        <v>10</v>
+        <v>33</v>
       </c>
       <c r="S357" s="5">
-        <v>11</v>
+        <v>35</v>
       </c>
       <c r="T357" s="3" t="s">
         <v>894</v>
@@ -47884,7 +47884,7 @@
         <v>46</v>
       </c>
       <c r="AA357" s="7">
-        <v>156000</v>
+        <v>339000</v>
       </c>
       <c r="AB357" s="7">
         <v>31</v>
@@ -47955,13 +47955,13 @@
         <v>951</v>
       </c>
       <c r="I358" s="3" t="s">
-        <v>909</v>
+        <v>912</v>
       </c>
       <c r="J358" s="3" t="s">
-        <v>910</v>
+        <v>913</v>
       </c>
       <c r="K358" s="3" t="s">
-        <v>911</v>
+        <v>914</v>
       </c>
       <c r="L358" s="3" t="s">
         <v>50</v>
@@ -48092,22 +48092,22 @@
         <v>50</v>
       </c>
       <c r="M359" s="3" t="s">
-        <v>62</v>
+        <v>131</v>
       </c>
       <c r="N359" s="3" t="s">
-        <v>63</v>
+        <v>132</v>
       </c>
       <c r="O359" s="3" t="s">
-        <v>64</v>
+        <v>133</v>
       </c>
       <c r="P359" s="3" t="s">
-        <v>65</v>
+        <v>134</v>
       </c>
       <c r="Q359" s="5">
         <v>2</v>
       </c>
       <c r="R359" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S359" s="5">
         <v>2</v>
@@ -48134,7 +48134,7 @@
         <v>46</v>
       </c>
       <c r="AA359" s="7">
-        <v>1211240</v>
+        <v>646676</v>
       </c>
       <c r="AB359" s="7">
         <v>1</v>
@@ -48205,37 +48205,37 @@
         <v>45</v>
       </c>
       <c r="I360" s="3" t="s">
-        <v>958</v>
+        <v>109</v>
       </c>
       <c r="J360" s="3" t="s">
-        <v>959</v>
+        <v>110</v>
       </c>
       <c r="K360" s="3" t="s">
-        <v>960</v>
+        <v>111</v>
       </c>
       <c r="L360" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M360" s="3" t="s">
-        <v>105</v>
+        <v>62</v>
       </c>
       <c r="N360" s="3" t="s">
-        <v>106</v>
+        <v>63</v>
       </c>
       <c r="O360" s="3" t="s">
-        <v>107</v>
+        <v>64</v>
       </c>
       <c r="P360" s="3" t="s">
-        <v>108</v>
+        <v>65</v>
       </c>
       <c r="Q360" s="5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R360" s="5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S360" s="5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T360" s="3" t="s">
         <v>894</v>
@@ -48259,7 +48259,7 @@
         <v>46</v>
       </c>
       <c r="AA360" s="7">
-        <v>663000</v>
+        <v>558000</v>
       </c>
       <c r="AB360" s="7">
         <v>1</v>
@@ -48286,10 +48286,10 @@
         <v>0</v>
       </c>
       <c r="AJ360" s="3" t="s">
-        <v>58</v>
+        <v>924</v>
       </c>
       <c r="AK360" s="6">
-        <v>46304.905077118055</v>
+        <v>46296.93825494213</v>
       </c>
       <c r="AL360" s="3" t="s">
         <v>46</v>
@@ -48298,10 +48298,10 @@
         <v>46</v>
       </c>
       <c r="AN360" s="3" t="s">
-        <v>58</v>
+        <v>924</v>
       </c>
       <c r="AO360" s="6">
-        <v>46304.905077118055</v>
+        <v>46296.93825494213</v>
       </c>
     </row>
     <row r="361" spans="1:41" x14ac:dyDescent="0.25">
@@ -48330,37 +48330,37 @@
         <v>45</v>
       </c>
       <c r="I361" s="3" t="s">
-        <v>286</v>
+        <v>135</v>
       </c>
       <c r="J361" s="3" t="s">
-        <v>287</v>
+        <v>136</v>
       </c>
       <c r="K361" s="3" t="s">
-        <v>288</v>
+        <v>137</v>
       </c>
       <c r="L361" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M361" s="3" t="s">
-        <v>105</v>
+        <v>131</v>
       </c>
       <c r="N361" s="3" t="s">
-        <v>106</v>
+        <v>132</v>
       </c>
       <c r="O361" s="3" t="s">
-        <v>107</v>
+        <v>133</v>
       </c>
       <c r="P361" s="3" t="s">
-        <v>108</v>
+        <v>134</v>
       </c>
       <c r="Q361" s="5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R361" s="5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S361" s="5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T361" s="3" t="s">
         <v>894</v>
@@ -48383,8 +48383,8 @@
       <c r="Z361" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="AA361" s="3" t="s">
-        <v>46</v>
+      <c r="AA361" s="7">
+        <v>536250</v>
       </c>
       <c r="AB361" s="7">
         <v>1</v>
@@ -48411,10 +48411,10 @@
         <v>0</v>
       </c>
       <c r="AJ361" s="3" t="s">
-        <v>58</v>
+        <v>924</v>
       </c>
       <c r="AK361" s="6">
-        <v>46301.927933530096</v>
+        <v>46296.93825494213</v>
       </c>
       <c r="AL361" s="3" t="s">
         <v>46</v>
@@ -48423,10 +48423,10 @@
         <v>46</v>
       </c>
       <c r="AN361" s="3" t="s">
-        <v>58</v>
+        <v>924</v>
       </c>
       <c r="AO361" s="6">
-        <v>46301.927933530096</v>
+        <v>46296.93825494213</v>
       </c>
     </row>
     <row r="362" spans="1:41" x14ac:dyDescent="0.25">
@@ -48455,28 +48455,28 @@
         <v>45</v>
       </c>
       <c r="I362" s="3" t="s">
-        <v>292</v>
+        <v>144</v>
       </c>
       <c r="J362" s="3" t="s">
-        <v>293</v>
+        <v>145</v>
       </c>
       <c r="K362" s="3" t="s">
-        <v>294</v>
+        <v>146</v>
       </c>
       <c r="L362" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M362" s="3" t="s">
-        <v>62</v>
+        <v>98</v>
       </c>
       <c r="N362" s="3" t="s">
-        <v>63</v>
+        <v>99</v>
       </c>
       <c r="O362" s="3" t="s">
-        <v>64</v>
+        <v>100</v>
       </c>
       <c r="P362" s="3" t="s">
-        <v>65</v>
+        <v>101</v>
       </c>
       <c r="Q362" s="5">
         <v>2</v>
@@ -48509,7 +48509,7 @@
         <v>46</v>
       </c>
       <c r="AA362" s="7">
-        <v>87000</v>
+        <v>2736757</v>
       </c>
       <c r="AB362" s="7">
         <v>1</v>
@@ -48580,28 +48580,28 @@
         <v>45</v>
       </c>
       <c r="I363" s="3" t="s">
-        <v>728</v>
+        <v>958</v>
       </c>
       <c r="J363" s="3" t="s">
-        <v>729</v>
+        <v>959</v>
       </c>
       <c r="K363" s="3" t="s">
-        <v>730</v>
+        <v>960</v>
       </c>
       <c r="L363" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M363" s="3" t="s">
-        <v>131</v>
+        <v>62</v>
       </c>
       <c r="N363" s="3" t="s">
-        <v>132</v>
+        <v>63</v>
       </c>
       <c r="O363" s="3" t="s">
-        <v>133</v>
+        <v>64</v>
       </c>
       <c r="P363" s="3" t="s">
-        <v>134</v>
+        <v>65</v>
       </c>
       <c r="Q363" s="5">
         <v>2</v>
@@ -48634,7 +48634,7 @@
         <v>46</v>
       </c>
       <c r="AA363" s="7">
-        <v>1567312</v>
+        <v>1211240</v>
       </c>
       <c r="AB363" s="7">
         <v>1</v>
@@ -48705,13 +48705,13 @@
         <v>45</v>
       </c>
       <c r="I364" s="3" t="s">
-        <v>322</v>
+        <v>961</v>
       </c>
       <c r="J364" s="3" t="s">
-        <v>323</v>
+        <v>962</v>
       </c>
       <c r="K364" s="3" t="s">
-        <v>324</v>
+        <v>963</v>
       </c>
       <c r="L364" s="3" t="s">
         <v>50</v>
@@ -48729,13 +48729,13 @@
         <v>108</v>
       </c>
       <c r="Q364" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R364" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S364" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="T364" s="3" t="s">
         <v>894</v>
@@ -48759,7 +48759,7 @@
         <v>46</v>
       </c>
       <c r="AA364" s="7">
-        <v>5131620</v>
+        <v>663000</v>
       </c>
       <c r="AB364" s="7">
         <v>1</v>
@@ -48786,10 +48786,10 @@
         <v>0</v>
       </c>
       <c r="AJ364" s="3" t="s">
-        <v>924</v>
+        <v>58</v>
       </c>
       <c r="AK364" s="6">
-        <v>46296.93825494213</v>
+        <v>46304.905077118055</v>
       </c>
       <c r="AL364" s="3" t="s">
         <v>46</v>
@@ -48798,10 +48798,10 @@
         <v>46</v>
       </c>
       <c r="AN364" s="3" t="s">
-        <v>924</v>
+        <v>58</v>
       </c>
       <c r="AO364" s="6">
-        <v>46296.93825494213</v>
+        <v>46304.905077118055</v>
       </c>
     </row>
     <row r="365" spans="1:41" x14ac:dyDescent="0.25">
@@ -48830,28 +48830,28 @@
         <v>45</v>
       </c>
       <c r="I365" s="3" t="s">
-        <v>422</v>
+        <v>722</v>
       </c>
       <c r="J365" s="3" t="s">
-        <v>423</v>
+        <v>723</v>
       </c>
       <c r="K365" s="3" t="s">
-        <v>424</v>
+        <v>724</v>
       </c>
       <c r="L365" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M365" s="3" t="s">
-        <v>131</v>
+        <v>62</v>
       </c>
       <c r="N365" s="3" t="s">
-        <v>132</v>
+        <v>63</v>
       </c>
       <c r="O365" s="3" t="s">
-        <v>133</v>
+        <v>64</v>
       </c>
       <c r="P365" s="3" t="s">
-        <v>134</v>
+        <v>65</v>
       </c>
       <c r="Q365" s="5">
         <v>2</v>
@@ -48884,7 +48884,7 @@
         <v>46</v>
       </c>
       <c r="AA365" s="7">
-        <v>698000</v>
+        <v>1227480</v>
       </c>
       <c r="AB365" s="7">
         <v>1</v>
@@ -48955,37 +48955,37 @@
         <v>45</v>
       </c>
       <c r="I366" s="3" t="s">
-        <v>772</v>
+        <v>286</v>
       </c>
       <c r="J366" s="3" t="s">
-        <v>773</v>
+        <v>287</v>
       </c>
       <c r="K366" s="3" t="s">
-        <v>774</v>
+        <v>288</v>
       </c>
       <c r="L366" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M366" s="3" t="s">
-        <v>62</v>
+        <v>105</v>
       </c>
       <c r="N366" s="3" t="s">
-        <v>63</v>
+        <v>106</v>
       </c>
       <c r="O366" s="3" t="s">
-        <v>64</v>
+        <v>107</v>
       </c>
       <c r="P366" s="3" t="s">
-        <v>65</v>
+        <v>108</v>
       </c>
       <c r="Q366" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R366" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S366" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="T366" s="3" t="s">
         <v>894</v>
@@ -49008,8 +49008,8 @@
       <c r="Z366" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="AA366" s="7">
-        <v>2482921</v>
+      <c r="AA366" s="3" t="s">
+        <v>46</v>
       </c>
       <c r="AB366" s="7">
         <v>1</v>
@@ -49036,10 +49036,10 @@
         <v>0</v>
       </c>
       <c r="AJ366" s="3" t="s">
-        <v>924</v>
+        <v>58</v>
       </c>
       <c r="AK366" s="6">
-        <v>46296.93825494213</v>
+        <v>46301.927933530096</v>
       </c>
       <c r="AL366" s="3" t="s">
         <v>46</v>
@@ -49048,10 +49048,10 @@
         <v>46</v>
       </c>
       <c r="AN366" s="3" t="s">
-        <v>924</v>
+        <v>58</v>
       </c>
       <c r="AO366" s="6">
-        <v>46296.93825494213</v>
+        <v>46301.927933530096</v>
       </c>
     </row>
     <row r="367" spans="1:41" x14ac:dyDescent="0.25">
@@ -49080,28 +49080,28 @@
         <v>45</v>
       </c>
       <c r="I367" s="3" t="s">
-        <v>464</v>
+        <v>292</v>
       </c>
       <c r="J367" s="3" t="s">
-        <v>465</v>
+        <v>293</v>
       </c>
       <c r="K367" s="3" t="s">
-        <v>466</v>
+        <v>294</v>
       </c>
       <c r="L367" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M367" s="3" t="s">
-        <v>125</v>
+        <v>62</v>
       </c>
       <c r="N367" s="3" t="s">
-        <v>126</v>
+        <v>63</v>
       </c>
       <c r="O367" s="3" t="s">
-        <v>127</v>
+        <v>64</v>
       </c>
       <c r="P367" s="3" t="s">
-        <v>128</v>
+        <v>65</v>
       </c>
       <c r="Q367" s="5">
         <v>2</v>
@@ -49134,7 +49134,7 @@
         <v>46</v>
       </c>
       <c r="AA367" s="7">
-        <v>1156433</v>
+        <v>87000</v>
       </c>
       <c r="AB367" s="7">
         <v>1</v>
@@ -49205,28 +49205,28 @@
         <v>45</v>
       </c>
       <c r="I368" s="3" t="s">
-        <v>473</v>
+        <v>728</v>
       </c>
       <c r="J368" s="3" t="s">
-        <v>474</v>
+        <v>729</v>
       </c>
       <c r="K368" s="3" t="s">
-        <v>475</v>
+        <v>730</v>
       </c>
       <c r="L368" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M368" s="3" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="N368" s="3" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="O368" s="3" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="P368" s="3" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="Q368" s="5">
         <v>2</v>
@@ -49259,7 +49259,7 @@
         <v>46</v>
       </c>
       <c r="AA368" s="7">
-        <v>839166</v>
+        <v>1567312</v>
       </c>
       <c r="AB368" s="7">
         <v>1</v>
@@ -49330,28 +49330,28 @@
         <v>45</v>
       </c>
       <c r="I369" s="3" t="s">
-        <v>961</v>
+        <v>929</v>
       </c>
       <c r="J369" s="3" t="s">
-        <v>962</v>
+        <v>930</v>
       </c>
       <c r="K369" s="3" t="s">
-        <v>963</v>
+        <v>931</v>
       </c>
       <c r="L369" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M369" s="3" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="N369" s="3" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="O369" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="P369" s="3" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="Q369" s="5">
         <v>2</v>
@@ -49384,7 +49384,7 @@
         <v>46</v>
       </c>
       <c r="AA369" s="7">
-        <v>771000</v>
+        <v>3025200</v>
       </c>
       <c r="AB369" s="7">
         <v>1</v>
@@ -49461,31 +49461,31 @@
         <v>965</v>
       </c>
       <c r="K370" s="3" t="s">
-        <v>966</v>
+        <v>813</v>
       </c>
       <c r="L370" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M370" s="3" t="s">
-        <v>105</v>
+        <v>131</v>
       </c>
       <c r="N370" s="3" t="s">
-        <v>106</v>
+        <v>132</v>
       </c>
       <c r="O370" s="3" t="s">
-        <v>107</v>
+        <v>133</v>
       </c>
       <c r="P370" s="3" t="s">
-        <v>108</v>
+        <v>134</v>
       </c>
       <c r="Q370" s="5">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="R370" s="5">
         <v>2</v>
       </c>
       <c r="S370" s="5">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="T370" s="3" t="s">
         <v>894</v>
@@ -49509,7 +49509,7 @@
         <v>46</v>
       </c>
       <c r="AA370" s="7">
-        <v>744240</v>
+        <v>468000</v>
       </c>
       <c r="AB370" s="7">
         <v>1</v>
@@ -49580,13 +49580,13 @@
         <v>45</v>
       </c>
       <c r="I371" s="3" t="s">
-        <v>925</v>
+        <v>322</v>
       </c>
       <c r="J371" s="3" t="s">
-        <v>926</v>
+        <v>323</v>
       </c>
       <c r="K371" s="3" t="s">
-        <v>927</v>
+        <v>324</v>
       </c>
       <c r="L371" s="3" t="s">
         <v>50</v>
@@ -49633,8 +49633,8 @@
       <c r="Z371" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="AA371" s="3" t="s">
-        <v>46</v>
+      <c r="AA371" s="7">
+        <v>5131620</v>
       </c>
       <c r="AB371" s="7">
         <v>1</v>
@@ -49705,37 +49705,37 @@
         <v>45</v>
       </c>
       <c r="I372" s="3" t="s">
-        <v>393</v>
+        <v>740</v>
       </c>
       <c r="J372" s="3" t="s">
-        <v>394</v>
+        <v>741</v>
       </c>
       <c r="K372" s="3" t="s">
-        <v>395</v>
+        <v>742</v>
       </c>
       <c r="L372" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M372" s="3" t="s">
-        <v>105</v>
+        <v>69</v>
       </c>
       <c r="N372" s="3" t="s">
-        <v>106</v>
+        <v>70</v>
       </c>
       <c r="O372" s="3" t="s">
-        <v>107</v>
+        <v>71</v>
       </c>
       <c r="P372" s="3" t="s">
-        <v>108</v>
+        <v>72</v>
       </c>
       <c r="Q372" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R372" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S372" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="T372" s="3" t="s">
         <v>894</v>
@@ -49759,7 +49759,7 @@
         <v>46</v>
       </c>
       <c r="AA372" s="7">
-        <v>692000</v>
+        <v>87000</v>
       </c>
       <c r="AB372" s="7">
         <v>1</v>
@@ -49786,10 +49786,10 @@
         <v>0</v>
       </c>
       <c r="AJ372" s="3" t="s">
-        <v>58</v>
+        <v>924</v>
       </c>
       <c r="AK372" s="6">
-        <v>46302.79881820602</v>
+        <v>46296.93825494213</v>
       </c>
       <c r="AL372" s="3" t="s">
         <v>46</v>
@@ -49798,10 +49798,10 @@
         <v>46</v>
       </c>
       <c r="AN372" s="3" t="s">
-        <v>58</v>
+        <v>924</v>
       </c>
       <c r="AO372" s="6">
-        <v>46302.79881820602</v>
+        <v>46296.93825494213</v>
       </c>
     </row>
     <row r="373" spans="1:41" x14ac:dyDescent="0.25">
@@ -49955,37 +49955,37 @@
         <v>45</v>
       </c>
       <c r="I374" s="3" t="s">
-        <v>740</v>
+        <v>393</v>
       </c>
       <c r="J374" s="3" t="s">
-        <v>741</v>
+        <v>394</v>
       </c>
       <c r="K374" s="3" t="s">
-        <v>742</v>
+        <v>395</v>
       </c>
       <c r="L374" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M374" s="3" t="s">
-        <v>69</v>
+        <v>105</v>
       </c>
       <c r="N374" s="3" t="s">
-        <v>70</v>
+        <v>106</v>
       </c>
       <c r="O374" s="3" t="s">
-        <v>71</v>
+        <v>107</v>
       </c>
       <c r="P374" s="3" t="s">
-        <v>72</v>
+        <v>108</v>
       </c>
       <c r="Q374" s="5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R374" s="5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S374" s="5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T374" s="3" t="s">
         <v>894</v>
@@ -50009,7 +50009,7 @@
         <v>46</v>
       </c>
       <c r="AA374" s="7">
-        <v>87000</v>
+        <v>692000</v>
       </c>
       <c r="AB374" s="7">
         <v>1</v>
@@ -50036,10 +50036,10 @@
         <v>0</v>
       </c>
       <c r="AJ374" s="3" t="s">
-        <v>924</v>
+        <v>58</v>
       </c>
       <c r="AK374" s="6">
-        <v>46296.93825494213</v>
+        <v>46302.79881820602</v>
       </c>
       <c r="AL374" s="3" t="s">
         <v>46</v>
@@ -50048,10 +50048,10 @@
         <v>46</v>
       </c>
       <c r="AN374" s="3" t="s">
-        <v>924</v>
+        <v>58</v>
       </c>
       <c r="AO374" s="6">
-        <v>46296.93825494213</v>
+        <v>46302.79881820602</v>
       </c>
     </row>
     <row r="375" spans="1:41" x14ac:dyDescent="0.25">
@@ -50080,37 +50080,37 @@
         <v>45</v>
       </c>
       <c r="I375" s="3" t="s">
-        <v>967</v>
+        <v>925</v>
       </c>
       <c r="J375" s="3" t="s">
-        <v>968</v>
+        <v>926</v>
       </c>
       <c r="K375" s="3" t="s">
-        <v>813</v>
+        <v>927</v>
       </c>
       <c r="L375" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M375" s="3" t="s">
-        <v>131</v>
+        <v>105</v>
       </c>
       <c r="N375" s="3" t="s">
-        <v>132</v>
+        <v>106</v>
       </c>
       <c r="O375" s="3" t="s">
-        <v>133</v>
+        <v>107</v>
       </c>
       <c r="P375" s="3" t="s">
-        <v>134</v>
+        <v>108</v>
       </c>
       <c r="Q375" s="5">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="R375" s="5">
         <v>2</v>
       </c>
       <c r="S375" s="5">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="T375" s="3" t="s">
         <v>894</v>
@@ -50133,8 +50133,8 @@
       <c r="Z375" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="AA375" s="7">
-        <v>468000</v>
+      <c r="AA375" s="3" t="s">
+        <v>46</v>
       </c>
       <c r="AB375" s="7">
         <v>1</v>
@@ -50205,28 +50205,28 @@
         <v>45</v>
       </c>
       <c r="I376" s="3" t="s">
-        <v>929</v>
+        <v>966</v>
       </c>
       <c r="J376" s="3" t="s">
-        <v>930</v>
+        <v>967</v>
       </c>
       <c r="K376" s="3" t="s">
-        <v>931</v>
+        <v>968</v>
       </c>
       <c r="L376" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M376" s="3" t="s">
-        <v>125</v>
+        <v>105</v>
       </c>
       <c r="N376" s="3" t="s">
-        <v>126</v>
+        <v>106</v>
       </c>
       <c r="O376" s="3" t="s">
-        <v>127</v>
+        <v>107</v>
       </c>
       <c r="P376" s="3" t="s">
-        <v>128</v>
+        <v>108</v>
       </c>
       <c r="Q376" s="5">
         <v>2</v>
@@ -50259,7 +50259,7 @@
         <v>46</v>
       </c>
       <c r="AA376" s="7">
-        <v>3025200</v>
+        <v>744240</v>
       </c>
       <c r="AB376" s="7">
         <v>1</v>
@@ -50330,28 +50330,28 @@
         <v>45</v>
       </c>
       <c r="I377" s="3" t="s">
-        <v>722</v>
+        <v>969</v>
       </c>
       <c r="J377" s="3" t="s">
-        <v>723</v>
+        <v>970</v>
       </c>
       <c r="K377" s="3" t="s">
-        <v>724</v>
+        <v>971</v>
       </c>
       <c r="L377" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M377" s="3" t="s">
-        <v>62</v>
+        <v>131</v>
       </c>
       <c r="N377" s="3" t="s">
-        <v>63</v>
+        <v>132</v>
       </c>
       <c r="O377" s="3" t="s">
-        <v>64</v>
+        <v>133</v>
       </c>
       <c r="P377" s="3" t="s">
-        <v>65</v>
+        <v>134</v>
       </c>
       <c r="Q377" s="5">
         <v>2</v>
@@ -50384,7 +50384,7 @@
         <v>46</v>
       </c>
       <c r="AA377" s="7">
-        <v>1227480</v>
+        <v>771000</v>
       </c>
       <c r="AB377" s="7">
         <v>1</v>
@@ -50455,28 +50455,28 @@
         <v>45</v>
       </c>
       <c r="I378" s="3" t="s">
-        <v>144</v>
+        <v>422</v>
       </c>
       <c r="J378" s="3" t="s">
-        <v>145</v>
+        <v>423</v>
       </c>
       <c r="K378" s="3" t="s">
-        <v>146</v>
+        <v>424</v>
       </c>
       <c r="L378" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M378" s="3" t="s">
-        <v>98</v>
+        <v>131</v>
       </c>
       <c r="N378" s="3" t="s">
-        <v>99</v>
+        <v>132</v>
       </c>
       <c r="O378" s="3" t="s">
-        <v>100</v>
+        <v>133</v>
       </c>
       <c r="P378" s="3" t="s">
-        <v>101</v>
+        <v>134</v>
       </c>
       <c r="Q378" s="5">
         <v>2</v>
@@ -50509,7 +50509,7 @@
         <v>46</v>
       </c>
       <c r="AA378" s="7">
-        <v>2736757</v>
+        <v>698000</v>
       </c>
       <c r="AB378" s="7">
         <v>1</v>
@@ -50580,28 +50580,28 @@
         <v>45</v>
       </c>
       <c r="I379" s="3" t="s">
-        <v>135</v>
+        <v>772</v>
       </c>
       <c r="J379" s="3" t="s">
-        <v>136</v>
+        <v>773</v>
       </c>
       <c r="K379" s="3" t="s">
-        <v>137</v>
+        <v>774</v>
       </c>
       <c r="L379" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M379" s="3" t="s">
-        <v>131</v>
+        <v>62</v>
       </c>
       <c r="N379" s="3" t="s">
-        <v>132</v>
+        <v>63</v>
       </c>
       <c r="O379" s="3" t="s">
-        <v>133</v>
+        <v>64</v>
       </c>
       <c r="P379" s="3" t="s">
-        <v>134</v>
+        <v>65</v>
       </c>
       <c r="Q379" s="5">
         <v>2</v>
@@ -50634,7 +50634,7 @@
         <v>46</v>
       </c>
       <c r="AA379" s="7">
-        <v>536250</v>
+        <v>2482921</v>
       </c>
       <c r="AB379" s="7">
         <v>1</v>
@@ -50705,28 +50705,28 @@
         <v>45</v>
       </c>
       <c r="I380" s="3" t="s">
-        <v>109</v>
+        <v>464</v>
       </c>
       <c r="J380" s="3" t="s">
-        <v>110</v>
+        <v>465</v>
       </c>
       <c r="K380" s="3" t="s">
-        <v>111</v>
+        <v>466</v>
       </c>
       <c r="L380" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M380" s="3" t="s">
-        <v>62</v>
+        <v>125</v>
       </c>
       <c r="N380" s="3" t="s">
-        <v>63</v>
+        <v>126</v>
       </c>
       <c r="O380" s="3" t="s">
-        <v>64</v>
+        <v>127</v>
       </c>
       <c r="P380" s="3" t="s">
-        <v>65</v>
+        <v>128</v>
       </c>
       <c r="Q380" s="5">
         <v>2</v>
@@ -50759,7 +50759,7 @@
         <v>46</v>
       </c>
       <c r="AA380" s="7">
-        <v>558000</v>
+        <v>1156433</v>
       </c>
       <c r="AB380" s="7">
         <v>1</v>
@@ -50830,34 +50830,34 @@
         <v>45</v>
       </c>
       <c r="I381" s="3" t="s">
-        <v>969</v>
+        <v>473</v>
       </c>
       <c r="J381" s="3" t="s">
-        <v>970</v>
+        <v>474</v>
       </c>
       <c r="K381" s="3" t="s">
-        <v>971</v>
+        <v>475</v>
       </c>
       <c r="L381" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M381" s="3" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="N381" s="3" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="O381" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="P381" s="3" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="Q381" s="5">
         <v>2</v>
       </c>
       <c r="R381" s="5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S381" s="5">
         <v>2</v>
@@ -50884,7 +50884,7 @@
         <v>46</v>
       </c>
       <c r="AA381" s="7">
-        <v>646676</v>
+        <v>839166</v>
       </c>
       <c r="AB381" s="7">
         <v>1</v>
@@ -50967,16 +50967,16 @@
         <v>50</v>
       </c>
       <c r="M382" s="3" t="s">
-        <v>125</v>
+        <v>105</v>
       </c>
       <c r="N382" s="3" t="s">
-        <v>126</v>
+        <v>106</v>
       </c>
       <c r="O382" s="3" t="s">
-        <v>127</v>
+        <v>107</v>
       </c>
       <c r="P382" s="3" t="s">
-        <v>128</v>
+        <v>108</v>
       </c>
       <c r="Q382" s="5">
         <v>2</v>
@@ -51009,7 +51009,7 @@
         <v>46</v>
       </c>
       <c r="AA382" s="7">
-        <v>362000</v>
+        <v>384000</v>
       </c>
       <c r="AB382" s="7">
         <v>1</v>
@@ -51217,16 +51217,16 @@
         <v>50</v>
       </c>
       <c r="M384" s="3" t="s">
-        <v>105</v>
+        <v>125</v>
       </c>
       <c r="N384" s="3" t="s">
-        <v>106</v>
+        <v>126</v>
       </c>
       <c r="O384" s="3" t="s">
-        <v>107</v>
+        <v>127</v>
       </c>
       <c r="P384" s="3" t="s">
-        <v>108</v>
+        <v>128</v>
       </c>
       <c r="Q384" s="5">
         <v>2</v>
@@ -51259,7 +51259,7 @@
         <v>46</v>
       </c>
       <c r="AA384" s="7">
-        <v>384000</v>
+        <v>362000</v>
       </c>
       <c r="AB384" s="7">
         <v>1</v>
@@ -52455,13 +52455,13 @@
         <v>45</v>
       </c>
       <c r="I394" s="3" t="s">
-        <v>909</v>
+        <v>912</v>
       </c>
       <c r="J394" s="3" t="s">
-        <v>910</v>
+        <v>913</v>
       </c>
       <c r="K394" s="3" t="s">
-        <v>911</v>
+        <v>914</v>
       </c>
       <c r="L394" s="3" t="s">
         <v>50</v>
@@ -53205,13 +53205,13 @@
         <v>45</v>
       </c>
       <c r="I400" s="3" t="s">
-        <v>915</v>
+        <v>900</v>
       </c>
       <c r="J400" s="3" t="s">
-        <v>916</v>
+        <v>901</v>
       </c>
       <c r="K400" s="3" t="s">
-        <v>917</v>
+        <v>902</v>
       </c>
       <c r="L400" s="3" t="s">
         <v>50</v>
@@ -55205,10 +55205,10 @@
         <v>999</v>
       </c>
       <c r="I416" s="3" t="s">
-        <v>967</v>
+        <v>964</v>
       </c>
       <c r="J416" s="3" t="s">
-        <v>968</v>
+        <v>965</v>
       </c>
       <c r="K416" s="3" t="s">
         <v>813</v>
@@ -60205,13 +60205,13 @@
         <v>921</v>
       </c>
       <c r="I456" s="3" t="s">
-        <v>915</v>
+        <v>900</v>
       </c>
       <c r="J456" s="3" t="s">
-        <v>916</v>
+        <v>901</v>
       </c>
       <c r="K456" s="3" t="s">
-        <v>917</v>
+        <v>902</v>
       </c>
       <c r="L456" s="3" t="s">
         <v>50</v>
@@ -61455,13 +61455,13 @@
         <v>45</v>
       </c>
       <c r="I466" s="3" t="s">
-        <v>969</v>
+        <v>955</v>
       </c>
       <c r="J466" s="3" t="s">
-        <v>970</v>
+        <v>956</v>
       </c>
       <c r="K466" s="3" t="s">
-        <v>971</v>
+        <v>957</v>
       </c>
       <c r="L466" s="3" t="s">
         <v>50</v>
@@ -62705,10 +62705,10 @@
         <v>45</v>
       </c>
       <c r="I476" s="3" t="s">
-        <v>967</v>
+        <v>964</v>
       </c>
       <c r="J476" s="3" t="s">
-        <v>968</v>
+        <v>965</v>
       </c>
       <c r="K476" s="3" t="s">
         <v>813</v>

</xml_diff>

<commit_message>
Auto sync Onetech 29/10/2026 07:52
</commit_message>
<xml_diff>
--- a/data/Thang10/DANH_SACH_KET_QUA_CUA_HANG_THAM_GIA_CHUONG_TRINH.xlsx
+++ b/data/Thang10/DANH_SACH_KET_QUA_CUA_HANG_THAM_GIA_CHUONG_TRINH.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15371" uniqueCount="1039">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15369" uniqueCount="1039">
   <si>
     <t>DANH_SACH_KET_QUA_CUA_HANG_THAM_GIA_CHUONG_TRINH</t>
   </si>
@@ -43383,8 +43383,8 @@
       <c r="Z321" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="AA321" s="3" t="s">
-        <v>46</v>
+      <c r="AA321" s="7">
+        <v>388301</v>
       </c>
       <c r="AB321" s="7">
         <v>31</v>
@@ -43732,7 +43732,7 @@
         <v>10</v>
       </c>
       <c r="R324" s="5">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="S324" s="5">
         <v>10</v>
@@ -43979,13 +43979,13 @@
         <v>82</v>
       </c>
       <c r="Q326" s="5">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="R326" s="5">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="S326" s="5">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="T326" s="3" t="s">
         <v>894</v>
@@ -44104,13 +44104,13 @@
         <v>72</v>
       </c>
       <c r="Q327" s="5">
+        <v>31</v>
+      </c>
+      <c r="R327" s="5">
         <v>30</v>
       </c>
-      <c r="R327" s="5">
-        <v>29</v>
-      </c>
       <c r="S327" s="5">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="T327" s="3" t="s">
         <v>894</v>
@@ -44354,13 +44354,13 @@
         <v>128</v>
       </c>
       <c r="Q329" s="5">
+        <v>27</v>
+      </c>
+      <c r="R329" s="5">
         <v>26</v>
       </c>
-      <c r="R329" s="5">
-        <v>25</v>
-      </c>
       <c r="S329" s="5">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="T329" s="3" t="s">
         <v>894</v>
@@ -45104,13 +45104,13 @@
         <v>128</v>
       </c>
       <c r="Q335" s="5">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="R335" s="5">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="S335" s="5">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="T335" s="3" t="s">
         <v>894</v>
@@ -45854,13 +45854,13 @@
         <v>128</v>
       </c>
       <c r="Q341" s="5">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="R341" s="5">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="S341" s="5">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="T341" s="3" t="s">
         <v>894</v>
@@ -45979,13 +45979,13 @@
         <v>72</v>
       </c>
       <c r="Q342" s="5">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R342" s="5">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="S342" s="5">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="T342" s="3" t="s">
         <v>894</v>
@@ -46729,13 +46729,13 @@
         <v>134</v>
       </c>
       <c r="Q348" s="5">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="R348" s="5">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="S348" s="5">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="T348" s="3" t="s">
         <v>894</v>
@@ -47104,13 +47104,13 @@
         <v>128</v>
       </c>
       <c r="Q351" s="5">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="R351" s="5">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="S351" s="5">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="T351" s="3" t="s">
         <v>894</v>
@@ -47604,13 +47604,13 @@
         <v>128</v>
       </c>
       <c r="Q355" s="5">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="R355" s="5">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="S355" s="5">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="T355" s="3" t="s">
         <v>894</v>
@@ -47729,13 +47729,13 @@
         <v>72</v>
       </c>
       <c r="Q356" s="5">
+        <v>30</v>
+      </c>
+      <c r="R356" s="5">
         <v>29</v>
       </c>
-      <c r="R356" s="5">
-        <v>28</v>
-      </c>
       <c r="S356" s="5">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="T356" s="3" t="s">
         <v>894</v>
@@ -48509,7 +48509,7 @@
         <v>46</v>
       </c>
       <c r="AA362" s="7">
-        <v>2736757</v>
+        <v>3118775</v>
       </c>
       <c r="AB362" s="7">
         <v>1</v>
@@ -51979,13 +51979,13 @@
         <v>72</v>
       </c>
       <c r="Q390" s="5">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R390" s="5">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="S390" s="5">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="T390" s="3" t="s">
         <v>894</v>
@@ -52229,13 +52229,13 @@
         <v>128</v>
       </c>
       <c r="Q392" s="5">
+        <v>29</v>
+      </c>
+      <c r="R392" s="5">
         <v>28</v>
       </c>
-      <c r="R392" s="5">
-        <v>27</v>
-      </c>
       <c r="S392" s="5">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="T392" s="3" t="s">
         <v>894</v>
@@ -52384,7 +52384,7 @@
         <v>46</v>
       </c>
       <c r="AA393" s="7">
-        <v>2736757</v>
+        <v>3118775</v>
       </c>
       <c r="AB393" s="7">
         <v>31</v>
@@ -53104,13 +53104,13 @@
         <v>128</v>
       </c>
       <c r="Q399" s="5">
+        <v>28</v>
+      </c>
+      <c r="R399" s="5">
         <v>27</v>
       </c>
-      <c r="R399" s="5">
-        <v>26</v>
-      </c>
       <c r="S399" s="5">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="T399" s="3" t="s">
         <v>894</v>
@@ -53259,7 +53259,7 @@
         <v>46</v>
       </c>
       <c r="AA400" s="7">
-        <v>20517221</v>
+        <v>39525221</v>
       </c>
       <c r="AB400" s="7">
         <v>31</v>
@@ -54104,13 +54104,13 @@
         <v>128</v>
       </c>
       <c r="Q407" s="5">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="R407" s="5">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="S407" s="5">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="T407" s="3" t="s">
         <v>894</v>
@@ -54979,13 +54979,13 @@
         <v>128</v>
       </c>
       <c r="Q414" s="5">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="R414" s="5">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="S414" s="5">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="T414" s="3" t="s">
         <v>894</v>
@@ -55104,13 +55104,13 @@
         <v>72</v>
       </c>
       <c r="Q415" s="5">
+        <v>32</v>
+      </c>
+      <c r="R415" s="5">
         <v>31</v>
       </c>
-      <c r="R415" s="5">
-        <v>30</v>
-      </c>
       <c r="S415" s="5">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="T415" s="3" t="s">
         <v>894</v>
@@ -55604,13 +55604,13 @@
         <v>134</v>
       </c>
       <c r="Q419" s="5">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="R419" s="5">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="S419" s="5">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="T419" s="3" t="s">
         <v>894</v>
@@ -55884,7 +55884,7 @@
         <v>46</v>
       </c>
       <c r="AA421" s="7">
-        <v>2156236</v>
+        <v>2434791</v>
       </c>
       <c r="AB421" s="7">
         <v>31</v>
@@ -57229,13 +57229,13 @@
         <v>128</v>
       </c>
       <c r="Q432" s="5">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="R432" s="5">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="S432" s="5">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="T432" s="3" t="s">
         <v>894</v>
@@ -57354,13 +57354,13 @@
         <v>72</v>
       </c>
       <c r="Q433" s="5">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="R433" s="5">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="S433" s="5">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="T433" s="3" t="s">
         <v>894</v>
@@ -57479,13 +57479,13 @@
         <v>54</v>
       </c>
       <c r="Q434" s="5">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="R434" s="5">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="S434" s="5">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="T434" s="3" t="s">
         <v>894</v>
@@ -57854,13 +57854,13 @@
         <v>128</v>
       </c>
       <c r="Q437" s="5">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="R437" s="5">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="S437" s="5">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="T437" s="3" t="s">
         <v>894</v>
@@ -58354,13 +58354,13 @@
         <v>54</v>
       </c>
       <c r="Q441" s="5">
+        <v>31</v>
+      </c>
+      <c r="R441" s="5">
         <v>30</v>
       </c>
-      <c r="R441" s="5">
-        <v>29</v>
-      </c>
       <c r="S441" s="5">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="T441" s="3" t="s">
         <v>894</v>
@@ -59854,13 +59854,13 @@
         <v>128</v>
       </c>
       <c r="Q453" s="5">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="R453" s="5">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="S453" s="5">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="T453" s="3" t="s">
         <v>894</v>
@@ -60259,7 +60259,7 @@
         <v>46</v>
       </c>
       <c r="AA456" s="7">
-        <v>15155995</v>
+        <v>22791835</v>
       </c>
       <c r="AB456" s="7">
         <v>31</v>
@@ -61008,8 +61008,8 @@
       <c r="Z462" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="AA462" s="3" t="s">
-        <v>46</v>
+      <c r="AA462" s="7">
+        <v>1103427</v>
       </c>
       <c r="AB462" s="7">
         <v>31</v>
@@ -61229,13 +61229,13 @@
         <v>72</v>
       </c>
       <c r="Q464" s="5">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R464" s="5">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="S464" s="5">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="T464" s="3" t="s">
         <v>894</v>
@@ -61604,13 +61604,13 @@
         <v>128</v>
       </c>
       <c r="Q467" s="5">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="R467" s="5">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="S467" s="5">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="T467" s="3" t="s">
         <v>894</v>
@@ -61979,13 +61979,13 @@
         <v>54</v>
       </c>
       <c r="Q470" s="5">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="R470" s="5">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="S470" s="5">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="T470" s="3" t="s">
         <v>894</v>
@@ -62979,13 +62979,13 @@
         <v>134</v>
       </c>
       <c r="Q478" s="5">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="R478" s="5">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="S478" s="5">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="T478" s="3" t="s">
         <v>894</v>
@@ -63104,13 +63104,13 @@
         <v>72</v>
       </c>
       <c r="Q479" s="5">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="R479" s="5">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="S479" s="5">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="T479" s="3" t="s">
         <v>894</v>
@@ -63354,13 +63354,13 @@
         <v>72</v>
       </c>
       <c r="Q481" s="5">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="R481" s="5">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="S481" s="5">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="T481" s="3" t="s">
         <v>894</v>

</xml_diff>

<commit_message>
Auto sync Onetech 30/10/2026 13:32
</commit_message>
<xml_diff>
--- a/data/Thang10/DANH_SACH_KET_QUA_CUA_HANG_THAM_GIA_CHUONG_TRINH.xlsx
+++ b/data/Thang10/DANH_SACH_KET_QUA_CUA_HANG_THAM_GIA_CHUONG_TRINH.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15339" uniqueCount="1039">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15330" uniqueCount="1039">
   <si>
     <t>DANH_SACH_KET_QUA_CUA_HANG_THAM_GIA_CHUONG_TRINH</t>
   </si>
@@ -6603,14 +6603,14 @@
       <c r="P27" s="3" t="s">
         <v>156</v>
       </c>
-      <c r="Q27" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="R27" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="S27" s="3" t="s">
-        <v>46</v>
+      <c r="Q27" s="5">
+        <v>1</v>
+      </c>
+      <c r="R27" s="5">
+        <v>1</v>
+      </c>
+      <c r="S27" s="5">
+        <v>1</v>
       </c>
       <c r="T27" s="3" t="s">
         <v>46</v>
@@ -7478,14 +7478,14 @@
       <c r="P34" s="3" t="s">
         <v>156</v>
       </c>
-      <c r="Q34" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="R34" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="S34" s="3" t="s">
-        <v>46</v>
+      <c r="Q34" s="5">
+        <v>1</v>
+      </c>
+      <c r="R34" s="5">
+        <v>1</v>
+      </c>
+      <c r="S34" s="5">
+        <v>1</v>
       </c>
       <c r="T34" s="3" t="s">
         <v>46</v>
@@ -11728,14 +11728,14 @@
       <c r="P68" s="3" t="s">
         <v>156</v>
       </c>
-      <c r="Q68" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="R68" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="S68" s="3" t="s">
-        <v>46</v>
+      <c r="Q68" s="5">
+        <v>1</v>
+      </c>
+      <c r="R68" s="3">
+        <v>0</v>
+      </c>
+      <c r="S68" s="5">
+        <v>1</v>
       </c>
       <c r="T68" s="3" t="s">
         <v>46</v>
@@ -44104,13 +44104,13 @@
         <v>72</v>
       </c>
       <c r="Q327" s="5">
+        <v>32</v>
+      </c>
+      <c r="R327" s="5">
         <v>31</v>
       </c>
-      <c r="R327" s="5">
-        <v>30</v>
-      </c>
       <c r="S327" s="5">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="T327" s="3" t="s">
         <v>885</v>
@@ -44479,13 +44479,13 @@
         <v>128</v>
       </c>
       <c r="Q330" s="5">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="R330" s="5">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="S330" s="5">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="T330" s="3" t="s">
         <v>885</v>
@@ -44604,13 +44604,13 @@
         <v>128</v>
       </c>
       <c r="Q331" s="5">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="R331" s="5">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="S331" s="5">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="T331" s="3" t="s">
         <v>885</v>
@@ -45979,13 +45979,13 @@
         <v>72</v>
       </c>
       <c r="Q342" s="5">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="R342" s="5">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="S342" s="5">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="T342" s="3" t="s">
         <v>885</v>
@@ -46104,13 +46104,13 @@
         <v>128</v>
       </c>
       <c r="Q343" s="5">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="R343" s="5">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="S343" s="5">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="T343" s="3" t="s">
         <v>885</v>
@@ -47729,13 +47729,13 @@
         <v>72</v>
       </c>
       <c r="Q356" s="5">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R356" s="5">
         <v>29</v>
       </c>
       <c r="S356" s="5">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="T356" s="3" t="s">
         <v>885</v>
@@ -51979,13 +51979,13 @@
         <v>72</v>
       </c>
       <c r="Q390" s="5">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="R390" s="5">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="S390" s="5">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="T390" s="3" t="s">
         <v>885</v>
@@ -55104,13 +55104,13 @@
         <v>72</v>
       </c>
       <c r="Q415" s="5">
+        <v>33</v>
+      </c>
+      <c r="R415" s="5">
         <v>32</v>
       </c>
-      <c r="R415" s="5">
-        <v>31</v>
-      </c>
       <c r="S415" s="5">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="T415" s="3" t="s">
         <v>885</v>
@@ -57354,13 +57354,13 @@
         <v>72</v>
       </c>
       <c r="Q433" s="5">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="R433" s="5">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="S433" s="5">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="T433" s="3" t="s">
         <v>885</v>
@@ -58354,13 +58354,13 @@
         <v>54</v>
       </c>
       <c r="Q441" s="5">
+        <v>34</v>
+      </c>
+      <c r="R441" s="5">
         <v>33</v>
       </c>
-      <c r="R441" s="5">
-        <v>32</v>
-      </c>
       <c r="S441" s="5">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="T441" s="3" t="s">
         <v>885</v>
@@ -59229,13 +59229,13 @@
         <v>128</v>
       </c>
       <c r="Q448" s="5">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="R448" s="5">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="S448" s="5">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="T448" s="3" t="s">
         <v>885</v>
@@ -61229,13 +61229,13 @@
         <v>72</v>
       </c>
       <c r="Q464" s="5">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="R464" s="5">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="S464" s="5">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="T464" s="3" t="s">
         <v>885</v>
@@ -61979,13 +61979,13 @@
         <v>54</v>
       </c>
       <c r="Q470" s="5">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="R470" s="5">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="S470" s="5">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="T470" s="3" t="s">
         <v>885</v>
@@ -62479,13 +62479,13 @@
         <v>128</v>
       </c>
       <c r="Q474" s="5">
+        <v>21</v>
+      </c>
+      <c r="R474" s="5">
         <v>19</v>
       </c>
-      <c r="R474" s="5">
-        <v>18</v>
-      </c>
       <c r="S474" s="5">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="T474" s="3" t="s">
         <v>885</v>
@@ -63104,13 +63104,13 @@
         <v>72</v>
       </c>
       <c r="Q479" s="5">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="R479" s="5">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="S479" s="5">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="T479" s="3" t="s">
         <v>885</v>

</xml_diff>

<commit_message>
Auto sync Onetech 31/10/2026 11:00
</commit_message>
<xml_diff>
--- a/data/Thang10/DANH_SACH_KET_QUA_CUA_HANG_THAM_GIA_CHUONG_TRINH.xlsx
+++ b/data/Thang10/DANH_SACH_KET_QUA_CUA_HANG_THAM_GIA_CHUONG_TRINH.xlsx
@@ -53229,13 +53229,13 @@
         <v>118</v>
       </c>
       <c r="Q400" s="5">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="R400" s="5">
         <v>9</v>
       </c>
       <c r="S400" s="5">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="T400" s="3" t="s">
         <v>879</v>
@@ -53354,13 +53354,13 @@
         <v>54</v>
       </c>
       <c r="Q401" s="5">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="R401" s="5">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="S401" s="5">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="T401" s="3" t="s">
         <v>879</v>
@@ -54729,13 +54729,13 @@
         <v>118</v>
       </c>
       <c r="Q412" s="5">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="R412" s="5">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="S412" s="5">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="T412" s="3" t="s">
         <v>879</v>
@@ -57729,13 +57729,13 @@
         <v>82</v>
       </c>
       <c r="Q436" s="5">
+        <v>14</v>
+      </c>
+      <c r="R436" s="5">
         <v>13</v>
       </c>
-      <c r="R436" s="5">
-        <v>12</v>
-      </c>
       <c r="S436" s="5">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="T436" s="3" t="s">
         <v>879</v>
@@ -58854,13 +58854,13 @@
         <v>118</v>
       </c>
       <c r="Q445" s="5">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="R445" s="5">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="S445" s="5">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="T445" s="3" t="s">
         <v>879</v>
@@ -58979,13 +58979,13 @@
         <v>54</v>
       </c>
       <c r="Q446" s="5">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="R446" s="5">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="S446" s="5">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="T446" s="3" t="s">
         <v>879</v>
@@ -59729,13 +59729,13 @@
         <v>82</v>
       </c>
       <c r="Q452" s="5">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="R452" s="5">
         <v>6</v>
       </c>
       <c r="S452" s="5">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T452" s="3" t="s">
         <v>879</v>
@@ -60354,13 +60354,13 @@
         <v>101</v>
       </c>
       <c r="Q457" s="5">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="R457" s="5">
         <v>13</v>
       </c>
       <c r="S457" s="5">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="T457" s="3" t="s">
         <v>879</v>
@@ -60729,13 +60729,13 @@
         <v>118</v>
       </c>
       <c r="Q460" s="5">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="R460" s="5">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="S460" s="5">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="T460" s="3" t="s">
         <v>879</v>
@@ -62854,13 +62854,13 @@
         <v>108</v>
       </c>
       <c r="Q477" s="5">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="R477" s="5">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S477" s="5">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T477" s="3" t="s">
         <v>879</v>
@@ -63229,13 +63229,13 @@
         <v>128</v>
       </c>
       <c r="Q480" s="5">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="R480" s="5">
         <v>9</v>
       </c>
       <c r="S480" s="5">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="T480" s="3" t="s">
         <v>879</v>
@@ -63354,13 +63354,13 @@
         <v>72</v>
       </c>
       <c r="Q481" s="5">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="R481" s="5">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="S481" s="5">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="T481" s="3" t="s">
         <v>879</v>

</xml_diff>

<commit_message>
Auto sync Onetech 31/10/2026 12:35
</commit_message>
<xml_diff>
--- a/data/Thang10/DANH_SACH_KET_QUA_CUA_HANG_THAM_GIA_CHUONG_TRINH.xlsx
+++ b/data/Thang10/DANH_SACH_KET_QUA_CUA_HANG_THAM_GIA_CHUONG_TRINH.xlsx
@@ -56979,13 +56979,13 @@
         <v>54</v>
       </c>
       <c r="Q430" s="5">
+        <v>36</v>
+      </c>
+      <c r="R430" s="5">
         <v>35</v>
       </c>
-      <c r="R430" s="5">
-        <v>34</v>
-      </c>
       <c r="S430" s="5">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="T430" s="3" t="s">
         <v>879</v>
@@ -61979,13 +61979,13 @@
         <v>54</v>
       </c>
       <c r="Q470" s="5">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="R470" s="5">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="S470" s="5">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="T470" s="3" t="s">
         <v>879</v>

</xml_diff>

<commit_message>
Auto sync Onetech 31/10/2026 14:30
</commit_message>
<xml_diff>
--- a/data/Thang10/DANH_SACH_KET_QUA_CUA_HANG_THAM_GIA_CHUONG_TRINH.xlsx
+++ b/data/Thang10/DANH_SACH_KET_QUA_CUA_HANG_THAM_GIA_CHUONG_TRINH.xlsx
@@ -44854,13 +44854,13 @@
         <v>128</v>
       </c>
       <c r="Q333" s="5">
+        <v>33</v>
+      </c>
+      <c r="R333" s="5">
         <v>32</v>
       </c>
-      <c r="R333" s="5">
-        <v>31</v>
-      </c>
       <c r="S333" s="5">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="T333" s="3" t="s">
         <v>879</v>
@@ -53729,13 +53729,13 @@
         <v>128</v>
       </c>
       <c r="Q404" s="5">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="R404" s="5">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="S404" s="5">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="T404" s="3" t="s">
         <v>879</v>
@@ -59479,13 +59479,13 @@
         <v>128</v>
       </c>
       <c r="Q450" s="5">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="R450" s="5">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="S450" s="5">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="T450" s="3" t="s">
         <v>879</v>

</xml_diff>

<commit_message>
Auto sync Onetech 31/10/2026 16:53
</commit_message>
<xml_diff>
--- a/data/Thang10/DANH_SACH_KET_QUA_CUA_HANG_THAM_GIA_CHUONG_TRINH.xlsx
+++ b/data/Thang10/DANH_SACH_KET_QUA_CUA_HANG_THAM_GIA_CHUONG_TRINH.xlsx
@@ -45979,13 +45979,13 @@
         <v>72</v>
       </c>
       <c r="Q342" s="5">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="R342" s="5">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="S342" s="5">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="T342" s="3" t="s">
         <v>879</v>

</xml_diff>

<commit_message>
Auto sync Onetech 31/10/2026 18:32
</commit_message>
<xml_diff>
--- a/data/Thang10/DANH_SACH_KET_QUA_CUA_HANG_THAM_GIA_CHUONG_TRINH.xlsx
+++ b/data/Thang10/DANH_SACH_KET_QUA_CUA_HANG_THAM_GIA_CHUONG_TRINH.xlsx
@@ -45729,13 +45729,13 @@
         <v>128</v>
       </c>
       <c r="Q340" s="5">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="R340" s="5">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="S340" s="5">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="T340" s="3" t="s">
         <v>879</v>
@@ -47604,13 +47604,13 @@
         <v>128</v>
       </c>
       <c r="Q355" s="5">
+        <v>30</v>
+      </c>
+      <c r="R355" s="5">
         <v>29</v>
       </c>
-      <c r="R355" s="5">
-        <v>28</v>
-      </c>
       <c r="S355" s="5">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="T355" s="3" t="s">
         <v>879</v>
@@ -47729,13 +47729,13 @@
         <v>128</v>
       </c>
       <c r="Q356" s="5">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="R356" s="5">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="S356" s="5">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="T356" s="3" t="s">
         <v>879</v>
@@ -54479,13 +54479,13 @@
         <v>128</v>
       </c>
       <c r="Q410" s="5">
+        <v>27</v>
+      </c>
+      <c r="R410" s="5">
         <v>26</v>
       </c>
-      <c r="R410" s="5">
-        <v>25</v>
-      </c>
       <c r="S410" s="5">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="T410" s="3" t="s">
         <v>879</v>
@@ -54604,13 +54604,13 @@
         <v>128</v>
       </c>
       <c r="Q411" s="5">
+        <v>21</v>
+      </c>
+      <c r="R411" s="5">
         <v>20</v>
       </c>
-      <c r="R411" s="5">
-        <v>19</v>
-      </c>
       <c r="S411" s="5">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="T411" s="3" t="s">
         <v>879</v>
@@ -60604,13 +60604,13 @@
         <v>128</v>
       </c>
       <c r="Q459" s="5">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="R459" s="5">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="S459" s="5">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="T459" s="3" t="s">
         <v>879</v>

</xml_diff>